<commit_message>
Added instructions up to 0C, updated document.
</commit_message>
<xml_diff>
--- a/Research/Instructions/Instructions Native SNES.xlsx
+++ b/Research/Instructions/Instructions Native SNES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Projects\BirdSNES\Research\Instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5937B94C-DF71-485F-AA68-22D953DB36C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAA89746-7FDA-4655-8BA9-E9CCA8B3EC2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$F$649</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$F$767</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="114">
   <si>
     <t>BRK (00)</t>
   </si>
@@ -92,6 +92,9 @@
     <t>Cycles: 3</t>
   </si>
   <si>
+    <t>Store as Address.</t>
+  </si>
+  <si>
     <t>ORA (05)</t>
   </si>
   <si>
@@ -116,6 +119,12 @@
     <t>Cycles: 4</t>
   </si>
   <si>
+    <t>Store as Address.L.</t>
+  </si>
+  <si>
+    <t>Absolute (Read/Modify/Write)</t>
+  </si>
+  <si>
     <t>Store as Pointer.</t>
   </si>
   <si>
@@ -2114,6 +2123,180 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> based off Operand.</t>
+    </r>
+  </si>
+  <si>
+    <t>PHD (0B)</t>
+  </si>
+  <si>
+    <r>
+      <t>Write to (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>-1)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Push </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>D</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.H onto stack.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Push </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>D</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L onto stack.</t>
+    </r>
+  </si>
+  <si>
+    <t>TSB (0C)</t>
+  </si>
+  <si>
+    <r>
+      <t>Read Address:</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>DB</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Read Address + 1:</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>DB</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Write to Address + 1:</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>DB</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Write to Address:</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>DB</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">If </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>M</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag is set, skip the next cycle.</t>
     </r>
   </si>
 </sst>
@@ -2138,7 +2321,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2166,6 +2349,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.749992370372631"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2286,7 +2481,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
@@ -2330,6 +2525,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -2339,19 +2535,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2686,7 +2883,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{236A51FB-68FA-4644-A8C6-D47AA32EBCC5}">
-  <dimension ref="B1:E602"/>
+  <dimension ref="B1:E731"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="4.7109375" customWidth="1"/>
@@ -2722,18 +2919,18 @@
         <v>4</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C4" s="14" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2742,7 +2939,7 @@
       </c>
       <c r="D5" s="9"/>
       <c r="E5" s="10" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2750,7 +2947,7 @@
         <v>1.2</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E6" s="10" t="s">
         <v>10</v>
@@ -2762,7 +2959,7 @@
       </c>
       <c r="D7" s="9"/>
       <c r="E7" s="10" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="8" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2770,10 +2967,10 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2788,10 +2985,10 @@
         <v>3.2</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2806,10 +3003,10 @@
         <v>4.2</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2818,35 +3015,35 @@
       </c>
       <c r="D13" s="9"/>
       <c r="E13" s="15" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C14" s="8"/>
       <c r="D14" s="9"/>
       <c r="E14" s="15" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C15" s="8"/>
       <c r="D15" s="9"/>
       <c r="E15" s="15" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C16" s="8"/>
       <c r="D16" s="9"/>
       <c r="E16" s="15" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="17" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C17" s="8"/>
       <c r="D17" s="9"/>
       <c r="E17" s="15" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2854,10 +3051,10 @@
         <v>5.2</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="19" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2866,7 +3063,7 @@
       </c>
       <c r="D19" s="9"/>
       <c r="E19" s="15" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="20" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2874,7 +3071,7 @@
         <v>6.2</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E20" s="15" t="s">
         <v>12</v>
@@ -2886,7 +3083,7 @@
       </c>
       <c r="D21" s="9"/>
       <c r="E21" s="15" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="22" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2894,7 +3091,7 @@
         <v>7.2</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="E22" s="15" t="s">
         <v>13</v>
@@ -2905,86 +3102,86 @@
         <v>8.1</v>
       </c>
       <c r="D23" s="10"/>
-      <c r="E23" s="20" t="s">
-        <v>64</v>
+      <c r="E23" s="21" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="24" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C24" s="11"/>
       <c r="D24" s="10"/>
-      <c r="E24" s="20"/>
+      <c r="E24" s="21"/>
     </row>
     <row r="25" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C25" s="8">
         <v>8.1999999999999993</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E25" s="10" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="26" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C26" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="D26" s="23"/>
-      <c r="E26" s="24"/>
+      <c r="C26" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="D26" s="24"/>
+      <c r="E26" s="25"/>
     </row>
     <row r="28" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="21" t="s">
+      <c r="B28" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="C28" s="21"/>
-      <c r="D28" s="21"/>
-      <c r="E28" s="21"/>
+      <c r="C28" s="22"/>
+      <c r="D28" s="22"/>
+      <c r="E28" s="22"/>
     </row>
     <row r="29" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="21"/>
-      <c r="C29" s="21"/>
-      <c r="D29" s="21"/>
-      <c r="E29" s="21"/>
+      <c r="B29" s="22"/>
+      <c r="C29" s="22"/>
+      <c r="D29" s="22"/>
+      <c r="E29" s="22"/>
     </row>
     <row r="30" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="21"/>
-      <c r="C30" s="21"/>
-      <c r="D30" s="21"/>
-      <c r="E30" s="21"/>
+      <c r="B30" s="22"/>
+      <c r="C30" s="22"/>
+      <c r="D30" s="22"/>
+      <c r="E30" s="22"/>
     </row>
     <row r="31" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="21"/>
-      <c r="C31" s="21"/>
-      <c r="D31" s="21"/>
-      <c r="E31" s="21"/>
+      <c r="B31" s="22"/>
+      <c r="C31" s="22"/>
+      <c r="D31" s="22"/>
+      <c r="E31" s="22"/>
     </row>
     <row r="32" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="21"/>
-      <c r="C32" s="21"/>
-      <c r="D32" s="21"/>
-      <c r="E32" s="21"/>
+      <c r="B32" s="22"/>
+      <c r="C32" s="22"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
     </row>
     <row r="33" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="21"/>
-      <c r="C33" s="21"/>
-      <c r="D33" s="21"/>
-      <c r="E33" s="21"/>
+      <c r="B33" s="22"/>
+      <c r="C33" s="22"/>
+      <c r="D33" s="22"/>
+      <c r="E33" s="22"/>
     </row>
     <row r="34" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="19" t="s">
-        <v>34</v>
-      </c>
-      <c r="C34" s="19"/>
-      <c r="D34" s="19"/>
-      <c r="E34" s="19"/>
+      <c r="B34" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="C34" s="20"/>
+      <c r="D34" s="20"/>
+      <c r="E34" s="20"/>
     </row>
     <row r="35" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="21" t="s">
-        <v>32</v>
-      </c>
-      <c r="C35" s="21"/>
-      <c r="D35" s="21"/>
-      <c r="E35" s="21"/>
+      <c r="B35" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="C35" s="22"/>
+      <c r="D35" s="22"/>
+      <c r="E35" s="22"/>
     </row>
     <row r="60" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C60" s="1" t="s">
@@ -3000,7 +3197,7 @@
     <row r="61" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C61" s="4"/>
       <c r="D61" s="5" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E61" s="6"/>
     </row>
@@ -3012,15 +3209,15 @@
         <v>4</v>
       </c>
       <c r="E62" s="7" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="63" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C63" s="14" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D63" s="12" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E63" s="12" t="s">
         <v>9</v>
@@ -3032,7 +3229,7 @@
       </c>
       <c r="D64" s="9"/>
       <c r="E64" s="10" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="65" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3040,10 +3237,10 @@
         <v>1.2</v>
       </c>
       <c r="D65" s="9" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E65" s="10" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="66" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3052,7 +3249,7 @@
       </c>
       <c r="D66" s="9"/>
       <c r="E66" s="10" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
     </row>
     <row r="67" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3061,7 +3258,7 @@
       </c>
       <c r="D67" s="9"/>
       <c r="E67" s="10" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="68" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3069,8 +3266,8 @@
         <v>3.1</v>
       </c>
       <c r="D68" s="17"/>
-      <c r="E68" s="26" t="s">
-        <v>35</v>
+      <c r="E68" s="27" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="69" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3078,7 +3275,7 @@
         <v>3.2</v>
       </c>
       <c r="D69" s="17"/>
-      <c r="E69" s="26"/>
+      <c r="E69" s="27"/>
     </row>
     <row r="70" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C70" s="8">
@@ -3095,7 +3292,7 @@
         <v>11</v>
       </c>
       <c r="E71" s="15" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="72" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3110,10 +3307,10 @@
         <v>5.2</v>
       </c>
       <c r="D73" s="9" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E73" s="15" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="74" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3124,14 +3321,14 @@
       <c r="E74" s="15"/>
     </row>
     <row r="75" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C75" s="8">
+      <c r="C75" s="19">
         <v>6.2</v>
       </c>
       <c r="D75" s="9" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E75" s="15" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="76" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3142,14 +3339,14 @@
       <c r="E76" s="18"/>
     </row>
     <row r="77" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C77" s="16">
+      <c r="C77" s="28">
         <v>7.2</v>
       </c>
       <c r="D77" s="17" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="E77" s="18" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="78" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3157,41 +3354,41 @@
         <v>8.1</v>
       </c>
       <c r="D78" s="9"/>
-      <c r="E78" s="20" t="s">
-        <v>95</v>
+      <c r="E78" s="21" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="79" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C79" s="8"/>
       <c r="D79" s="9"/>
-      <c r="E79" s="20"/>
+      <c r="E79" s="21"/>
     </row>
     <row r="80" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C80" s="8"/>
       <c r="D80" s="9"/>
-      <c r="E80" s="20"/>
+      <c r="E80" s="21"/>
     </row>
     <row r="81" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C81" s="8">
         <v>8.1999999999999993</v>
       </c>
       <c r="D81" s="9" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E81" s="15" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="82" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C82" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="D82" s="23"/>
-      <c r="E82" s="25"/>
+      <c r="C82" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="D82" s="24"/>
+      <c r="E82" s="26"/>
     </row>
     <row r="119" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C119" s="1" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D119" s="2" t="s">
         <v>15</v>
@@ -3215,15 +3412,15 @@
         <v>4</v>
       </c>
       <c r="E121" s="7" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="122" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C122" s="14" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D122" s="12" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E122" s="12" t="s">
         <v>9</v>
@@ -3235,7 +3432,7 @@
       </c>
       <c r="D123" s="9"/>
       <c r="E123" s="10" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="124" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3243,7 +3440,7 @@
         <v>1.2</v>
       </c>
       <c r="D124" s="9" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E124" s="10" t="s">
         <v>10</v>
@@ -3255,7 +3452,7 @@
       </c>
       <c r="D125" s="9"/>
       <c r="E125" s="10" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="126" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3263,10 +3460,10 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="D126" s="9" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E126" s="10" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="127" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3275,7 +3472,7 @@
       </c>
       <c r="D127" s="9"/>
       <c r="E127" s="10" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="128" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3283,10 +3480,10 @@
         <v>3.2</v>
       </c>
       <c r="D128" s="9" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="E128" s="10" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="129" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3301,10 +3498,10 @@
         <v>4.2</v>
       </c>
       <c r="D130" s="9" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="E130" s="15" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="131" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3313,7 +3510,7 @@
       </c>
       <c r="D131" s="9"/>
       <c r="E131" s="15" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="132" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3321,10 +3518,10 @@
         <v>5.2</v>
       </c>
       <c r="D132" s="9" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="E132" s="15" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="133" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3333,7 +3530,7 @@
       </c>
       <c r="D133" s="9"/>
       <c r="E133" s="15" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="134" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3341,7 +3538,7 @@
         <v>6.2</v>
       </c>
       <c r="D134" s="9" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E134" s="15" t="s">
         <v>12</v>
@@ -3353,15 +3550,15 @@
       </c>
       <c r="D135" s="9"/>
       <c r="E135" s="15" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="136" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C136" s="8">
+      <c r="C136" s="19">
         <v>7.2</v>
       </c>
       <c r="D136" s="9" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="E136" s="15" t="s">
         <v>13</v>
@@ -3372,85 +3569,85 @@
         <v>8.1</v>
       </c>
       <c r="D137" s="9"/>
-      <c r="E137" s="20" t="s">
-        <v>64</v>
+      <c r="E137" s="21" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="138" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C138" s="8"/>
       <c r="D138" s="9"/>
-      <c r="E138" s="20"/>
+      <c r="E138" s="21"/>
     </row>
     <row r="139" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C139" s="8">
         <v>8.1999999999999993</v>
       </c>
       <c r="D139" s="9" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E139" s="15" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="140" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C140" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="D140" s="23"/>
-      <c r="E140" s="25"/>
+      <c r="C140" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="D140" s="24"/>
+      <c r="E140" s="26"/>
     </row>
     <row r="142" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B142" s="21" t="s">
+      <c r="B142" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="C142" s="21"/>
-      <c r="D142" s="21"/>
-      <c r="E142" s="21"/>
+      <c r="C142" s="22"/>
+      <c r="D142" s="22"/>
+      <c r="E142" s="22"/>
     </row>
     <row r="143" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B143" s="21"/>
-      <c r="C143" s="21"/>
-      <c r="D143" s="21"/>
-      <c r="E143" s="21"/>
+      <c r="B143" s="22"/>
+      <c r="C143" s="22"/>
+      <c r="D143" s="22"/>
+      <c r="E143" s="22"/>
     </row>
     <row r="144" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B144" s="21"/>
-      <c r="C144" s="21"/>
-      <c r="D144" s="21"/>
-      <c r="E144" s="21"/>
+      <c r="B144" s="22"/>
+      <c r="C144" s="22"/>
+      <c r="D144" s="22"/>
+      <c r="E144" s="22"/>
     </row>
     <row r="145" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B145" s="21"/>
-      <c r="C145" s="21"/>
-      <c r="D145" s="21"/>
-      <c r="E145" s="21"/>
+      <c r="B145" s="22"/>
+      <c r="C145" s="22"/>
+      <c r="D145" s="22"/>
+      <c r="E145" s="22"/>
     </row>
     <row r="146" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B146" s="21"/>
-      <c r="C146" s="21"/>
-      <c r="D146" s="21"/>
-      <c r="E146" s="21"/>
+      <c r="B146" s="22"/>
+      <c r="C146" s="22"/>
+      <c r="D146" s="22"/>
+      <c r="E146" s="22"/>
     </row>
     <row r="147" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B147" s="21"/>
-      <c r="C147" s="21"/>
-      <c r="D147" s="21"/>
-      <c r="E147" s="21"/>
+      <c r="B147" s="22"/>
+      <c r="C147" s="22"/>
+      <c r="D147" s="22"/>
+      <c r="E147" s="22"/>
     </row>
     <row r="148" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B148" s="21" t="s">
-        <v>52</v>
-      </c>
-      <c r="C148" s="21"/>
-      <c r="D148" s="21"/>
-      <c r="E148" s="21"/>
+      <c r="B148" s="22" t="s">
+        <v>55</v>
+      </c>
+      <c r="C148" s="22"/>
+      <c r="D148" s="22"/>
+      <c r="E148" s="22"/>
     </row>
     <row r="178" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C178" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D178" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E178" s="3" t="s">
         <v>8</v>
@@ -3459,7 +3656,7 @@
     <row r="179" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C179" s="4"/>
       <c r="D179" s="5" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="E179" s="6"/>
     </row>
@@ -3471,15 +3668,15 @@
         <v>4</v>
       </c>
       <c r="E180" s="7" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="181" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C181" s="14" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D181" s="12" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E181" s="12" t="s">
         <v>9</v>
@@ -3491,7 +3688,7 @@
       </c>
       <c r="D182" s="9"/>
       <c r="E182" s="10" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="183" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3499,10 +3696,10 @@
         <v>1.2</v>
       </c>
       <c r="D183" s="9" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E183" s="10" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="184" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3511,7 +3708,7 @@
       </c>
       <c r="D184" s="9"/>
       <c r="E184" s="10" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="185" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3529,14 +3726,14 @@
       <c r="E186" s="10"/>
     </row>
     <row r="187" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C187" s="8">
+      <c r="C187" s="19">
         <v>3.2</v>
       </c>
       <c r="D187" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E187" s="10" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="188" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3547,14 +3744,14 @@
       <c r="E188" s="18"/>
     </row>
     <row r="189" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C189" s="16">
+      <c r="C189" s="28">
         <v>4.2</v>
       </c>
       <c r="D189" s="17" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E189" s="18" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="190" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3562,44 +3759,44 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="D190" s="9"/>
-      <c r="E190" s="20" t="s">
-        <v>95</v>
+      <c r="E190" s="21" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="191" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C191" s="8"/>
       <c r="D191" s="9"/>
-      <c r="E191" s="20"/>
+      <c r="E191" s="21"/>
     </row>
     <row r="192" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C192" s="8"/>
       <c r="D192" s="9"/>
-      <c r="E192" s="20"/>
+      <c r="E192" s="21"/>
     </row>
     <row r="193" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C193" s="8">
         <v>5.2</v>
       </c>
       <c r="D193" s="9" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E193" s="15" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="194" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C194" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="D194" s="23"/>
-      <c r="E194" s="25"/>
+      <c r="C194" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="D194" s="24"/>
+      <c r="E194" s="26"/>
     </row>
     <row r="237" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C237" s="1" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D237" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E237" s="3" t="s">
         <v>8</v>
@@ -3608,7 +3805,7 @@
     <row r="238" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C238" s="4"/>
       <c r="D238" s="5" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="E238" s="6"/>
     </row>
@@ -3620,15 +3817,15 @@
         <v>4</v>
       </c>
       <c r="E239" s="7" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="240" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C240" s="14" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D240" s="12" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E240" s="12" t="s">
         <v>9</v>
@@ -3640,7 +3837,7 @@
       </c>
       <c r="D241" s="9"/>
       <c r="E241" s="10" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="242" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3648,10 +3845,10 @@
         <v>1.2</v>
       </c>
       <c r="D242" s="9" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E242" s="10" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="243" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3659,8 +3856,8 @@
         <v>2.1</v>
       </c>
       <c r="D243" s="17"/>
-      <c r="E243" s="26" t="s">
-        <v>60</v>
+      <c r="E243" s="27" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="244" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3668,21 +3865,21 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="D244" s="17"/>
-      <c r="E244" s="26"/>
+      <c r="E244" s="27"/>
     </row>
     <row r="245" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C245" s="8">
         <v>3.1</v>
       </c>
       <c r="D245" s="9"/>
-      <c r="E245" s="20" t="s">
-        <v>82</v>
+      <c r="E245" s="21" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="246" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C246" s="8"/>
       <c r="D246" s="9"/>
-      <c r="E246" s="20"/>
+      <c r="E246" s="21"/>
     </row>
     <row r="247" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C247" s="8">
@@ -3692,7 +3889,7 @@
         <v>11</v>
       </c>
       <c r="E247" s="10" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="248" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3707,10 +3904,10 @@
         <v>4.2</v>
       </c>
       <c r="D249" s="17" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E249" s="18" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="250" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3718,19 +3915,19 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="D250" s="9"/>
-      <c r="E250" s="20" t="s">
-        <v>96</v>
+      <c r="E250" s="21" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="251" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C251" s="8"/>
       <c r="D251" s="9"/>
-      <c r="E251" s="20"/>
+      <c r="E251" s="21"/>
     </row>
     <row r="252" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C252" s="8"/>
       <c r="D252" s="9"/>
-      <c r="E252" s="20"/>
+      <c r="E252" s="21"/>
     </row>
     <row r="253" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C253" s="8">
@@ -3738,7 +3935,7 @@
       </c>
       <c r="D253" s="9"/>
       <c r="E253" s="15" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
     </row>
     <row r="254" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3753,10 +3950,10 @@
         <v>6.2</v>
       </c>
       <c r="D255" s="17" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E255" s="18" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="256" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3767,14 +3964,14 @@
       <c r="E256" s="15"/>
     </row>
     <row r="257" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C257" s="8">
+      <c r="C257" s="19">
         <v>7.2</v>
       </c>
       <c r="D257" s="9" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E257" s="15" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="258" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3789,22 +3986,22 @@
         <v>8.1999999999999993</v>
       </c>
       <c r="D259" s="9" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E259" s="15" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="260" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C260" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="D260" s="23"/>
-      <c r="E260" s="25"/>
+      <c r="C260" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="D260" s="24"/>
+      <c r="E260" s="26"/>
     </row>
     <row r="296" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C296" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D296" s="2" t="s">
         <v>16</v>
@@ -3816,7 +4013,7 @@
     <row r="297" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C297" s="4"/>
       <c r="D297" s="5" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="E297" s="6"/>
     </row>
@@ -3828,15 +4025,15 @@
         <v>4</v>
       </c>
       <c r="E298" s="7" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="299" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C299" s="14" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D299" s="12" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E299" s="12" t="s">
         <v>9</v>
@@ -3848,7 +4045,7 @@
       </c>
       <c r="D300" s="9"/>
       <c r="E300" s="10" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="301" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3856,10 +4053,10 @@
         <v>1.2</v>
       </c>
       <c r="D301" s="9" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E301" s="10" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="302" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3867,8 +4064,8 @@
         <v>2.1</v>
       </c>
       <c r="D302" s="17"/>
-      <c r="E302" s="26" t="s">
-        <v>60</v>
+      <c r="E302" s="27" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="303" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3876,31 +4073,31 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="D303" s="17"/>
-      <c r="E303" s="26"/>
+      <c r="E303" s="27"/>
     </row>
     <row r="304" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C304" s="8">
         <v>3.1</v>
       </c>
       <c r="D304" s="9"/>
-      <c r="E304" s="20" t="s">
-        <v>82</v>
+      <c r="E304" s="21" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="305" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C305" s="8"/>
       <c r="D305" s="9"/>
-      <c r="E305" s="20"/>
+      <c r="E305" s="21"/>
     </row>
     <row r="306" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C306" s="8">
+      <c r="C306" s="19">
         <v>3.2</v>
       </c>
       <c r="D306" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E306" s="15" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="307" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3908,17 +4105,17 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="D307" s="17"/>
-      <c r="E307" s="26"/>
+      <c r="E307" s="27"/>
     </row>
     <row r="308" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C308" s="16">
+      <c r="C308" s="28">
         <v>4.2</v>
       </c>
       <c r="D308" s="17" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E308" s="18" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="309" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3926,44 +4123,44 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="D309" s="9"/>
-      <c r="E309" s="20" t="s">
-        <v>95</v>
+      <c r="E309" s="21" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="310" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C310" s="8"/>
       <c r="D310" s="9"/>
-      <c r="E310" s="20"/>
+      <c r="E310" s="21"/>
     </row>
     <row r="311" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C311" s="8"/>
       <c r="D311" s="9"/>
-      <c r="E311" s="20"/>
+      <c r="E311" s="21"/>
     </row>
     <row r="312" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C312" s="8">
         <v>5.2</v>
       </c>
       <c r="D312" s="9" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E312" s="15" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="313" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C313" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="D313" s="23"/>
-      <c r="E313" s="25"/>
+      <c r="C313" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="D313" s="24"/>
+      <c r="E313" s="26"/>
     </row>
     <row r="355" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C355" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D355" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E355" s="3" t="s">
         <v>8</v>
@@ -3972,7 +4169,7 @@
     <row r="356" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C356" s="4"/>
       <c r="D356" s="5" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="E356" s="6"/>
     </row>
@@ -3984,15 +4181,15 @@
         <v>4</v>
       </c>
       <c r="E357" s="7" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="358" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C358" s="14" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D358" s="12" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E358" s="12" t="s">
         <v>9</v>
@@ -4004,7 +4201,7 @@
       </c>
       <c r="D359" s="9"/>
       <c r="E359" s="10" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="360" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4012,10 +4209,10 @@
         <v>1.2</v>
       </c>
       <c r="D360" s="9" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E360" s="10" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="361" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4023,8 +4220,8 @@
         <v>2.1</v>
       </c>
       <c r="D361" s="17"/>
-      <c r="E361" s="26" t="s">
-        <v>60</v>
+      <c r="E361" s="27" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="362" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4032,21 +4229,21 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="D362" s="17"/>
-      <c r="E362" s="26"/>
+      <c r="E362" s="27"/>
     </row>
     <row r="363" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C363" s="8">
         <v>3.1</v>
       </c>
       <c r="D363" s="9"/>
-      <c r="E363" s="20" t="s">
-        <v>82</v>
+      <c r="E363" s="21" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="364" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C364" s="8"/>
       <c r="D364" s="9"/>
-      <c r="E364" s="20"/>
+      <c r="E364" s="21"/>
     </row>
     <row r="365" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C365" s="8">
@@ -4056,7 +4253,7 @@
         <v>11</v>
       </c>
       <c r="E365" s="10" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="366" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4064,17 +4261,17 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="D366" s="17"/>
-      <c r="E366" s="26"/>
+      <c r="E366" s="27"/>
     </row>
     <row r="367" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C367" s="16">
         <v>4.2</v>
       </c>
       <c r="D367" s="17" t="s">
-        <v>38</v>
-      </c>
-      <c r="E367" s="26" t="s">
-        <v>39</v>
+        <v>41</v>
+      </c>
+      <c r="E367" s="27" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="368" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4082,29 +4279,29 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="D368" s="9"/>
-      <c r="E368" s="20" t="s">
-        <v>100</v>
+      <c r="E368" s="21" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="369" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C369" s="8"/>
       <c r="D369" s="9"/>
-      <c r="E369" s="20"/>
+      <c r="E369" s="21"/>
     </row>
     <row r="370" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C370" s="8"/>
       <c r="D370" s="9"/>
-      <c r="E370" s="20"/>
+      <c r="E370" s="21"/>
     </row>
     <row r="371" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C371" s="8"/>
       <c r="D371" s="9"/>
-      <c r="E371" s="20"/>
+      <c r="E371" s="21"/>
     </row>
     <row r="372" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C372" s="8"/>
       <c r="D372" s="9"/>
-      <c r="E372" s="20"/>
+      <c r="E372" s="21"/>
     </row>
     <row r="373" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C373" s="8">
@@ -4112,7 +4309,7 @@
       </c>
       <c r="D373" s="9"/>
       <c r="E373" s="15" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
     </row>
     <row r="374" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4120,17 +4317,17 @@
         <v>6.1</v>
       </c>
       <c r="D374" s="17"/>
-      <c r="E374" s="26"/>
+      <c r="E374" s="27"/>
     </row>
     <row r="375" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C375" s="16">
         <v>6.2</v>
       </c>
       <c r="D375" s="17" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E375" s="18" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="376" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4141,14 +4338,14 @@
       <c r="E376" s="10"/>
     </row>
     <row r="377" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C377" s="8">
+      <c r="C377" s="19">
         <v>7.2</v>
       </c>
       <c r="D377" s="9" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E377" s="10" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="378" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4163,22 +4360,22 @@
         <v>8.1999999999999993</v>
       </c>
       <c r="D379" s="9" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E379" s="15" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="380" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C380" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="D380" s="23"/>
-      <c r="E380" s="25"/>
+      <c r="C380" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="D380" s="24"/>
+      <c r="E380" s="26"/>
     </row>
     <row r="414" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C414" s="1" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D414" s="2" t="s">
         <v>7</v>
@@ -4190,7 +4387,7 @@
     <row r="415" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C415" s="4"/>
       <c r="D415" s="5" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="E415" s="6"/>
     </row>
@@ -4202,15 +4399,15 @@
         <v>4</v>
       </c>
       <c r="E416" s="7" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="417" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C417" s="14" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D417" s="12" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E417" s="12" t="s">
         <v>9</v>
@@ -4222,7 +4419,7 @@
       </c>
       <c r="D418" s="9"/>
       <c r="E418" s="10" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="419" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4230,10 +4427,10 @@
         <v>1.2</v>
       </c>
       <c r="D419" s="9" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E419" s="10" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="420" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4241,8 +4438,8 @@
         <v>2.1</v>
       </c>
       <c r="D420" s="17"/>
-      <c r="E420" s="26" t="s">
-        <v>60</v>
+      <c r="E420" s="27" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="421" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4250,21 +4447,21 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="D421" s="17"/>
-      <c r="E421" s="26"/>
+      <c r="E421" s="27"/>
     </row>
     <row r="422" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C422" s="8">
         <v>3.1</v>
       </c>
       <c r="D422" s="9"/>
-      <c r="E422" s="20" t="s">
-        <v>82</v>
+      <c r="E422" s="21" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="423" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C423" s="8"/>
       <c r="D423" s="9"/>
-      <c r="E423" s="20"/>
+      <c r="E423" s="21"/>
     </row>
     <row r="424" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C424" s="8">
@@ -4274,7 +4471,7 @@
         <v>11</v>
       </c>
       <c r="E424" s="15" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="425" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4289,10 +4486,10 @@
         <v>4.2</v>
       </c>
       <c r="D426" s="9" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E426" s="10" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="427" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4307,10 +4504,10 @@
         <v>5.2</v>
       </c>
       <c r="D428" s="9" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="E428" s="15" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="429" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4321,14 +4518,14 @@
       <c r="E429" s="15"/>
     </row>
     <row r="430" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C430" s="8">
+      <c r="C430" s="19">
         <v>6.2</v>
       </c>
       <c r="D430" s="9" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E430" s="15" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="431" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4339,14 +4536,14 @@
       <c r="E431" s="18"/>
     </row>
     <row r="432" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C432" s="16">
+      <c r="C432" s="28">
         <v>7.2</v>
       </c>
       <c r="D432" s="17" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E432" s="18" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="433" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4354,41 +4551,41 @@
         <v>8.1</v>
       </c>
       <c r="D433" s="9"/>
-      <c r="E433" s="20" t="s">
-        <v>95</v>
+      <c r="E433" s="21" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="434" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C434" s="8"/>
       <c r="D434" s="9"/>
-      <c r="E434" s="20"/>
+      <c r="E434" s="21"/>
     </row>
     <row r="435" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C435" s="8"/>
       <c r="D435" s="9"/>
-      <c r="E435" s="20"/>
+      <c r="E435" s="21"/>
     </row>
     <row r="436" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C436" s="8">
         <v>8.1999999999999993</v>
       </c>
       <c r="D436" s="9" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E436" s="15" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="437" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C437" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="D437" s="23"/>
-      <c r="E437" s="24"/>
+      <c r="C437" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="D437" s="24"/>
+      <c r="E437" s="25"/>
     </row>
     <row r="473" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C473" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D473" s="2" t="s">
         <v>16</v>
@@ -4412,15 +4609,15 @@
         <v>4</v>
       </c>
       <c r="E475" s="7" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="476" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C476" s="14" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D476" s="12" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E476" s="12" t="s">
         <v>9</v>
@@ -4432,7 +4629,7 @@
       </c>
       <c r="D477" s="9"/>
       <c r="E477" s="10" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="478" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4448,18 +4645,18 @@
       </c>
       <c r="D479" s="9"/>
       <c r="E479" s="10" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="480" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C480" s="8">
+      <c r="C480" s="19">
         <v>2.2000000000000002</v>
       </c>
       <c r="D480" s="9" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="E480" s="10" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="481" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4474,34 +4671,34 @@
         <v>3.2</v>
       </c>
       <c r="D482" s="9" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E482" s="10" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="483" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C483" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="D483" s="23"/>
-      <c r="E483" s="25"/>
+      <c r="C483" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="D483" s="24"/>
+      <c r="E483" s="26"/>
     </row>
     <row r="532" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C532" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D532" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E532" s="3" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="533" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C533" s="4"/>
       <c r="D533" s="5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E533" s="6"/>
     </row>
@@ -4513,15 +4710,15 @@
         <v>4</v>
       </c>
       <c r="E534" s="7" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="535" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C535" s="14" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D535" s="12" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E535" s="12" t="s">
         <v>9</v>
@@ -4533,18 +4730,18 @@
       </c>
       <c r="D536" s="9"/>
       <c r="E536" s="10" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="537" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C537" s="8">
+      <c r="C537" s="19">
         <v>1.2</v>
       </c>
       <c r="D537" s="9" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E537" s="10" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="538" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4552,19 +4749,19 @@
         <v>2.1</v>
       </c>
       <c r="D538" s="17"/>
-      <c r="E538" s="26" t="s">
-        <v>60</v>
+      <c r="E538" s="27" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="539" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C539" s="16">
+      <c r="C539" s="28">
         <v>2.2000000000000002</v>
       </c>
       <c r="D539" s="17" t="s">
-        <v>94</v>
-      </c>
-      <c r="E539" s="26" t="s">
-        <v>39</v>
+        <v>97</v>
+      </c>
+      <c r="E539" s="27" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="540" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4572,44 +4769,44 @@
         <v>3.1</v>
       </c>
       <c r="D540" s="9"/>
-      <c r="E540" s="20" t="s">
-        <v>97</v>
+      <c r="E540" s="21" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="541" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C541" s="8"/>
       <c r="D541" s="9"/>
-      <c r="E541" s="20"/>
+      <c r="E541" s="21"/>
     </row>
     <row r="542" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C542" s="8"/>
       <c r="D542" s="9"/>
-      <c r="E542" s="20"/>
+      <c r="E542" s="21"/>
     </row>
     <row r="543" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C543" s="8">
         <v>3.2</v>
       </c>
       <c r="D543" s="9" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E543" s="10" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="544" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C544" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="D544" s="23"/>
-      <c r="E544" s="25"/>
+      <c r="C544" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="D544" s="24"/>
+      <c r="E544" s="26"/>
     </row>
     <row r="591" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C591" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D591" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="D591" s="2" t="s">
-        <v>22</v>
       </c>
       <c r="E591" s="3" t="s">
         <v>14</v>
@@ -4630,15 +4827,15 @@
         <v>4</v>
       </c>
       <c r="E593" s="7" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="594" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C594" s="14" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D594" s="12" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E594" s="12" t="s">
         <v>9</v>
@@ -4650,18 +4847,18 @@
       </c>
       <c r="D595" s="9"/>
       <c r="E595" s="10" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="596" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C596" s="8">
+      <c r="C596" s="19">
         <v>1.2</v>
       </c>
       <c r="D596" s="9" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E596" s="10" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="597" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4669,46 +4866,371 @@
         <v>2.1</v>
       </c>
       <c r="D597" s="9"/>
-      <c r="E597" s="20" t="s">
-        <v>99</v>
+      <c r="E597" s="21" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="598" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C598" s="8"/>
       <c r="D598" s="9"/>
-      <c r="E598" s="20"/>
+      <c r="E598" s="21"/>
     </row>
     <row r="599" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C599" s="8"/>
       <c r="D599" s="9"/>
-      <c r="E599" s="20"/>
+      <c r="E599" s="21"/>
     </row>
     <row r="600" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C600" s="8"/>
       <c r="D600" s="9"/>
-      <c r="E600" s="20"/>
+      <c r="E600" s="21"/>
     </row>
     <row r="601" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C601" s="8">
         <v>2.2000000000000002</v>
       </c>
       <c r="D601" s="9" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E601" s="10" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="602" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C602" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="D602" s="23"/>
-      <c r="E602" s="25"/>
+      <c r="C602" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="D602" s="24"/>
+      <c r="E602" s="26"/>
+    </row>
+    <row r="650" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C650" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D650" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E650" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="651" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C651" s="4"/>
+      <c r="D651" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E651" s="6"/>
+    </row>
+    <row r="652" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C652" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="D652" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E652" s="7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="653" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C653" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="D653" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="E653" s="12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="654" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C654" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="D654" s="9"/>
+      <c r="E654" s="10" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="655" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C655" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="D655" s="9"/>
+      <c r="E655" s="10"/>
+    </row>
+    <row r="656" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C656" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="D656" s="9"/>
+      <c r="E656" s="10"/>
+    </row>
+    <row r="657" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C657" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="D657" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E657" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="658" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C658" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="D658" s="9"/>
+      <c r="E658" s="10"/>
+    </row>
+    <row r="659" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C659" s="19">
+        <v>3.2</v>
+      </c>
+      <c r="D659" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="E659" s="10" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="660" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C660" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="D660" s="9"/>
+      <c r="E660" s="15"/>
+    </row>
+    <row r="661" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C661" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="D661" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="E661" s="15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="662" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C662" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="D662" s="24"/>
+      <c r="E662" s="26"/>
+    </row>
+    <row r="709" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C709" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="D709" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E709" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="710" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C710" s="4"/>
+      <c r="D710" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E710" s="6"/>
+    </row>
+    <row r="711" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C711" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="D711" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E711" s="7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="712" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C712" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="D712" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="E712" s="12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="713" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C713" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="D713" s="9"/>
+      <c r="E713" s="10" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="714" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C714" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="D714" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="E714" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="715" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C715" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="D715" s="9"/>
+      <c r="E715" s="10" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="716" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C716" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="D716" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="E716" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="717" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C717" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="D717" s="9"/>
+      <c r="E717" s="10" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="718" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C718" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="D718" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="E718" s="10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="719" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C719" s="16">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="D719" s="17"/>
+      <c r="E719" s="18"/>
+    </row>
+    <row r="720" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C720" s="16">
+        <v>4.2</v>
+      </c>
+      <c r="D720" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="E720" s="18" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="721" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C721" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="D721" s="9"/>
+      <c r="E721" s="21" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="722" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C722" s="8"/>
+      <c r="D722" s="9"/>
+      <c r="E722" s="21"/>
+    </row>
+    <row r="723" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C723" s="8"/>
+      <c r="D723" s="9"/>
+      <c r="E723" s="21"/>
+    </row>
+    <row r="724" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C724" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="D724" s="9"/>
+      <c r="E724" s="15" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="725" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C725" s="16">
+        <v>6.1</v>
+      </c>
+      <c r="D725" s="17"/>
+      <c r="E725" s="18"/>
+    </row>
+    <row r="726" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C726" s="28">
+        <v>6.2</v>
+      </c>
+      <c r="D726" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="E726" s="18" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="727" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C727" s="8">
+        <v>7.1</v>
+      </c>
+      <c r="D727" s="9"/>
+      <c r="E727" s="15"/>
+    </row>
+    <row r="728" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C728" s="19">
+        <v>7.2</v>
+      </c>
+      <c r="D728" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="E728" s="15" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="729" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C729" s="8">
+        <v>8.1</v>
+      </c>
+      <c r="D729" s="9"/>
+      <c r="E729" s="10"/>
+    </row>
+    <row r="730" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C730" s="8">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="D730" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="E730" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="731" spans="3:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C731" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="D731" s="24"/>
+      <c r="E731" s="25"/>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="20">
     <mergeCell ref="E597:E600"/>
+    <mergeCell ref="E721:E723"/>
     <mergeCell ref="E23:E24"/>
     <mergeCell ref="E137:E138"/>
     <mergeCell ref="E190:E192"/>

</xml_diff>

<commit_message>
Added instructions up to 19.
</commit_message>
<xml_diff>
--- a/Research/Instructions/Instructions Native SNES.xlsx
+++ b/Research/Instructions/Instructions Native SNES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Projects\BirdSNES\Research\Instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD1CC2BF-6A0B-430E-BE97-9AB3660BE115}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F08A4A0D-695D-4359-AE48-4F2A75F6213C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$D$1357</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$D$1534</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="683" uniqueCount="159">
   <si>
     <t>BRK (00)</t>
   </si>
@@ -3016,6 +3016,102 @@
   </si>
   <si>
     <t>Direct Indexed Indirect (d,x) (Read/Modify/Write)</t>
+  </si>
+  <si>
+    <t>ORA (17)</t>
+  </si>
+  <si>
+    <t>Direct Indirect Indexed Long [d],y (Read)</t>
+  </si>
+  <si>
+    <t>CLC (18)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Sets the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag to 0.</t>
+    </r>
+  </si>
+  <si>
+    <t>ORA (19)</t>
+  </si>
+  <si>
+    <t>Absolute, Y (Read)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Inc. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. Perform Orig = Pointer.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Perform Tmp = ui32(Pointer + </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>).</t>
+    </r>
+  </si>
+  <si>
+    <t>Bank += (Tmp &gt;&gt; 16).</t>
   </si>
 </sst>
 </file>
@@ -3616,7 +3712,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{236A51FB-68FA-4644-A8C6-D47AA32EBCC5}">
-  <dimension ref="A1:D1323"/>
+  <dimension ref="A1:D1497"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.7109375" customWidth="1"/>
@@ -7703,9 +7799,508 @@
       <c r="C1323" s="21"/>
       <c r="D1323" s="23"/>
     </row>
+    <row r="1358" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1358" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="C1358" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1358" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="1359" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1359" s="4"/>
+      <c r="C1359" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="D1359" s="31"/>
+    </row>
+    <row r="1360" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1360" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1360" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1360" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1361" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1361" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1361" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1361" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1362" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1362" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C1362" s="9"/>
+      <c r="D1362" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1363" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1363" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="C1363" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1363" s="10" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="1364" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1364" s="16">
+        <v>2.1</v>
+      </c>
+      <c r="C1364" s="17"/>
+      <c r="D1364" s="24" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1365" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1365" s="16">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C1365" s="17"/>
+      <c r="D1365" s="24"/>
+    </row>
+    <row r="1366" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1366" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="C1366" s="9"/>
+      <c r="D1366" s="15" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="1367" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1367" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="C1367" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1367" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="1368" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1368" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="C1368" s="9"/>
+      <c r="D1368" s="15"/>
+    </row>
+    <row r="1369" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1369" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="C1369" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D1369" s="15" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="1370" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1370" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="C1370" s="9"/>
+      <c r="D1370" s="10"/>
+    </row>
+    <row r="1371" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1371" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="C1371" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="D1371" s="10" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="1372" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1372" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="C1372" s="9"/>
+      <c r="D1372" s="15" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="1373" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1373" s="8"/>
+      <c r="C1373" s="9"/>
+      <c r="D1373" s="15" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="1374" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1374" s="8"/>
+      <c r="C1374" s="9"/>
+      <c r="D1374" s="15" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="1375" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1375" s="19">
+        <v>6.2</v>
+      </c>
+      <c r="C1375" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="D1375" s="15" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="1376" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1376" s="16">
+        <v>7.1</v>
+      </c>
+      <c r="C1376" s="17"/>
+      <c r="D1376" s="18"/>
+    </row>
+    <row r="1377" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1377" s="25">
+        <v>7.2</v>
+      </c>
+      <c r="C1377" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="D1377" s="18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="1378" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1378" s="8">
+        <v>8.1</v>
+      </c>
+      <c r="C1378" s="9"/>
+      <c r="D1378" s="29" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="1379" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1379" s="8"/>
+      <c r="C1379" s="9"/>
+      <c r="D1379" s="29"/>
+    </row>
+    <row r="1380" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1380" s="8">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="C1380" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1380" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1381" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1381" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1381" s="21"/>
+      <c r="D1381" s="23"/>
+    </row>
+    <row r="1417" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1417" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C1417" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1417" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="1418" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1418" s="4"/>
+      <c r="C1418" s="26" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1418" s="27"/>
+    </row>
+    <row r="1419" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1419" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1419" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1419" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1420" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1420" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1420" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1420" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1421" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1421" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C1421" s="9"/>
+      <c r="D1421" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1422" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1422" s="19">
+        <v>1.2</v>
+      </c>
+      <c r="C1422" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1422" s="10" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="1423" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1423" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="C1423" s="9"/>
+      <c r="D1423" s="10" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="1424" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1424" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C1424" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1424" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1425" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1425" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1425" s="21"/>
+      <c r="D1425" s="23"/>
+    </row>
+    <row r="1476" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1476" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="C1476" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1476" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1477" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1477" s="4"/>
+      <c r="C1477" s="30" t="s">
+        <v>155</v>
+      </c>
+      <c r="D1477" s="31"/>
+    </row>
+    <row r="1478" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1478" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1478" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1478" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1479" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1479" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1479" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1479" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1480" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1480" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C1480" s="9"/>
+      <c r="D1480" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1481" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1481" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="C1481" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="D1481" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="1482" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1482" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="C1482" s="9"/>
+      <c r="D1482" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1483" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1483" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C1483" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="D1483" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="1484" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1484" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="C1484" s="9"/>
+      <c r="D1484" s="15" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="1485" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1485" s="8"/>
+      <c r="C1485" s="9"/>
+      <c r="D1485" s="15" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="1486" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1486" s="8"/>
+      <c r="C1486" s="9"/>
+      <c r="D1486" s="10" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="1487" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1487" s="8"/>
+      <c r="C1487" s="9"/>
+      <c r="D1487" s="10" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="1488" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1488" s="8"/>
+      <c r="C1488" s="9"/>
+      <c r="D1488" s="10" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="1489" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1489" s="16">
+        <v>3.2</v>
+      </c>
+      <c r="C1489" s="17"/>
+      <c r="D1489" s="24"/>
+    </row>
+    <row r="1490" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1490" s="16">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="C1490" s="17"/>
+      <c r="D1490" s="18"/>
+    </row>
+    <row r="1491" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1491" s="19">
+        <v>4.2</v>
+      </c>
+      <c r="C1491" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="D1491" s="15" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="1492" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1492" s="16">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="C1492" s="17"/>
+      <c r="D1492" s="24"/>
+    </row>
+    <row r="1493" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1493" s="25">
+        <v>5.2</v>
+      </c>
+      <c r="C1493" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="D1493" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="1494" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1494" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="C1494" s="9"/>
+      <c r="D1494" s="29" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="1495" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1495" s="8"/>
+      <c r="C1495" s="9"/>
+      <c r="D1495" s="29"/>
+    </row>
+    <row r="1496" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1496" s="8">
+        <v>6.2</v>
+      </c>
+      <c r="C1496" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="D1496" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1497" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1497" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1497" s="21"/>
+      <c r="D1497" s="23"/>
+    </row>
   </sheetData>
-  <mergeCells count="29">
+  <mergeCells count="33">
+    <mergeCell ref="C1477:D1477"/>
+    <mergeCell ref="D1494:D1495"/>
     <mergeCell ref="D1313:D1315"/>
+    <mergeCell ref="C1359:D1359"/>
+    <mergeCell ref="D1378:D1379"/>
     <mergeCell ref="D597:D599"/>
     <mergeCell ref="D721:D722"/>
     <mergeCell ref="C1300:D1300"/>

</xml_diff>

<commit_message>
Implemented/documented instructions up to 25.
</commit_message>
<xml_diff>
--- a/Research/Instructions/Instructions Native SNES.xlsx
+++ b/Research/Instructions/Instructions Native SNES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Projects\BirdSNES\Research\Instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F08A4A0D-695D-4359-AE48-4F2A75F6213C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4DB7F92-D5D9-4ED5-8638-5F18291E6BE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$D$1534</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$D$2220</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="683" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="995" uniqueCount="191">
   <si>
     <t>BRK (00)</t>
   </si>
@@ -3112,6 +3112,1073 @@
   </si>
   <si>
     <t>Bank += (Tmp &gt;&gt; 16).</t>
+  </si>
+  <si>
+    <t>INC (1A)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">If </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>M</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag is set, perform </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L += 1, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L &amp; $80), and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L, otherwise perform </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> += 1, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.H &amp; $80), and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>TSC (1B)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Sets </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>TRB (1C)</t>
+  </si>
+  <si>
+    <t>ORA (1D)</t>
+  </si>
+  <si>
+    <t>Absolute, X (Read)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Tmp = ui32(Pointer + </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>).</t>
+    </r>
+  </si>
+  <si>
+    <t>ASL (1E)</t>
+  </si>
+  <si>
+    <t>Absolute, X (Read/Modiy/Write)</t>
+  </si>
+  <si>
+    <t>Write to Pointer + 1:Bank</t>
+  </si>
+  <si>
+    <t>Write to Pointer:Bank</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Inc. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Perform Tmp = ui32(Pointer + </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>).</t>
+    </r>
+  </si>
+  <si>
+    <t>ORA (1F)</t>
+  </si>
+  <si>
+    <t>Absolute Long, X (Read)</t>
+  </si>
+  <si>
+    <t>JSR (20)</t>
+  </si>
+  <si>
+    <t>Absolute</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Dec. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> by 2. Perform </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> = Address.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Dec. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Discard, then schedule </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> -= 1.</t>
+    </r>
+  </si>
+  <si>
+    <t>AND (21)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Perform </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &amp;= Operand. If </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>M</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag is set, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L &amp; $80) and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L, otherwise set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.H &amp; $80) and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>JSL (22)</t>
+  </si>
+  <si>
+    <t>Absolute Long</t>
+  </si>
+  <si>
+    <r>
+      <t>Read (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>+0)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Write to (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>-2)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Inc </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Dec. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> by 3.  Copy Address to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Copy Bank to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PB</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>AND (23)</t>
+  </si>
+  <si>
+    <t>BIT (24)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">If </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>M</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag is set, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L &amp; Operand.L), set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (Operand.L &amp; $80), and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>V</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (Operand.L &amp; $40), otherwise set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &amp; Operand), set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (Operand.H &amp; $80), set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>V</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (Operand.H &amp; $40).</t>
+    </r>
+  </si>
+  <si>
+    <t>AND (25)</t>
   </si>
 </sst>
 </file>
@@ -3295,7 +4362,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
@@ -3377,6 +4444,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3712,7 +4782,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{236A51FB-68FA-4644-A8C6-D47AA32EBCC5}">
-  <dimension ref="A1:D1497"/>
+  <dimension ref="A1:D2199"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.7109375" customWidth="1"/>
@@ -8294,8 +9364,2030 @@
       <c r="C1497" s="21"/>
       <c r="D1497" s="23"/>
     </row>
+    <row r="1535" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1535" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="C1535" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1535" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="1536" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1536" s="4"/>
+      <c r="C1536" s="26" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1536" s="27"/>
+    </row>
+    <row r="1537" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1537" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1537" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1537" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1538" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1538" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1538" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1538" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1539" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1539" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C1539" s="9"/>
+      <c r="D1539" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1540" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1540" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="C1540" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1540" s="10" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="1541" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1541" s="19">
+        <v>2.1</v>
+      </c>
+      <c r="C1541" s="9"/>
+      <c r="D1541" s="29" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="1542" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1542" s="8"/>
+      <c r="C1542" s="9"/>
+      <c r="D1542" s="29"/>
+    </row>
+    <row r="1543" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1543" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C1543" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1543" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1544" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1544" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1544" s="21"/>
+      <c r="D1544" s="23"/>
+    </row>
+    <row r="1594" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1594" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="C1594" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1594" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="1595" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1595" s="4"/>
+      <c r="C1595" s="26" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1595" s="27"/>
+    </row>
+    <row r="1596" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1596" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1596" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1596" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1597" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1597" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1597" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1597" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1598" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1598" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C1598" s="9"/>
+      <c r="D1598" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1599" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1599" s="19">
+        <v>1.2</v>
+      </c>
+      <c r="C1599" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1599" s="10" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="1600" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1600" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="C1600" s="9"/>
+      <c r="D1600" s="10" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="1601" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1601" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C1601" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1601" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1602" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1602" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1602" s="21"/>
+      <c r="D1602" s="23"/>
+    </row>
+    <row r="1653" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1653" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C1653" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1653" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1654" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1654" s="4"/>
+      <c r="C1654" s="30" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1654" s="31"/>
+    </row>
+    <row r="1655" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1655" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1655" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1655" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1656" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1656" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1656" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1656" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1657" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1657" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C1657" s="9"/>
+      <c r="D1657" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1658" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1658" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="C1658" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1658" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="1659" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1659" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="C1659" s="9"/>
+      <c r="D1659" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1660" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1660" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C1660" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1660" s="10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="1661" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1661" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="C1661" s="9"/>
+      <c r="D1661" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1662" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1662" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="C1662" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="D1662" s="15" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="1663" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1663" s="16">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="C1663" s="17"/>
+      <c r="D1663" s="24"/>
+    </row>
+    <row r="1664" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1664" s="16">
+        <v>4.2</v>
+      </c>
+      <c r="C1664" s="17" t="s">
+        <v>106</v>
+      </c>
+      <c r="D1664" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="1665" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1665" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="C1665" s="9"/>
+      <c r="D1665" s="29" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="1666" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1666" s="8"/>
+      <c r="C1666" s="9"/>
+      <c r="D1666" s="29"/>
+    </row>
+    <row r="1667" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1667" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="C1667" s="9"/>
+      <c r="D1667" s="10" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="1668" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1668" s="16">
+        <v>6.1</v>
+      </c>
+      <c r="C1668" s="17"/>
+      <c r="D1668" s="18"/>
+    </row>
+    <row r="1669" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1669" s="16">
+        <v>6.2</v>
+      </c>
+      <c r="C1669" s="17" t="s">
+        <v>107</v>
+      </c>
+      <c r="D1669" s="18" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1670" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1670" s="8">
+        <v>7.1</v>
+      </c>
+      <c r="C1670" s="9"/>
+      <c r="D1670" s="10"/>
+    </row>
+    <row r="1671" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1671" s="19">
+        <v>7.2</v>
+      </c>
+      <c r="C1671" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="D1671" s="10" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="1672" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1672" s="8">
+        <v>8.1</v>
+      </c>
+      <c r="C1672" s="9"/>
+      <c r="D1672" s="10"/>
+    </row>
+    <row r="1673" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1673" s="8">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="C1673" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1673" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1674" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1674" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1674" s="21"/>
+      <c r="D1674" s="23"/>
+    </row>
+    <row r="1712" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1712" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="C1712" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1712" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1713" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1713" s="4"/>
+      <c r="C1713" s="26" t="s">
+        <v>165</v>
+      </c>
+      <c r="D1713" s="27"/>
+    </row>
+    <row r="1714" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1714" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1714" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1714" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1715" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1715" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1715" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1715" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1716" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1716" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C1716" s="9"/>
+      <c r="D1716" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1717" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1717" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="C1717" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="D1717" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="1718" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1718" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="C1718" s="9"/>
+      <c r="D1718" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1719" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1719" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C1719" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="D1719" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="1720" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1720" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="C1720" s="9"/>
+      <c r="D1720" s="10" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="1721" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1721" s="8"/>
+      <c r="C1721" s="9"/>
+      <c r="D1721" s="10" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="1722" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1722" s="8"/>
+      <c r="C1722" s="9"/>
+      <c r="D1722" s="10" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="1723" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1723" s="8"/>
+      <c r="C1723" s="9"/>
+      <c r="D1723" s="10" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="1724" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1724" s="8"/>
+      <c r="C1724" s="9"/>
+      <c r="D1724" s="10" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="1725" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1725" s="16">
+        <v>3.2</v>
+      </c>
+      <c r="C1725" s="17"/>
+      <c r="D1725" s="18"/>
+    </row>
+    <row r="1726" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1726" s="16">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="C1726" s="17"/>
+      <c r="D1726" s="24"/>
+    </row>
+    <row r="1727" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1727" s="19">
+        <v>4.2</v>
+      </c>
+      <c r="C1727" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="D1727" s="10" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="1728" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1728" s="16">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="C1728" s="17"/>
+      <c r="D1728" s="24"/>
+    </row>
+    <row r="1729" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1729" s="25">
+        <v>5.2</v>
+      </c>
+      <c r="C1729" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="D1729" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="1730" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1730" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="C1730" s="9"/>
+      <c r="D1730" s="29" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="1731" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1731" s="8"/>
+      <c r="C1731" s="9"/>
+      <c r="D1731" s="29"/>
+    </row>
+    <row r="1732" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1732" s="8">
+        <v>6.2</v>
+      </c>
+      <c r="C1732" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="D1732" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1733" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1733" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1733" s="21"/>
+      <c r="D1733" s="23"/>
+    </row>
+    <row r="1771" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1771" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C1771" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="D1771" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1772" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1772" s="4"/>
+      <c r="C1772" s="30" t="s">
+        <v>168</v>
+      </c>
+      <c r="D1772" s="31"/>
+    </row>
+    <row r="1773" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1773" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1773" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1773" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1774" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1774" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1774" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1774" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1775" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1775" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C1775" s="9"/>
+      <c r="D1775" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1776" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1776" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="C1776" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="D1776" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="1777" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1777" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="C1777" s="9"/>
+      <c r="D1777" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1778" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1778" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C1778" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="D1778" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="1779" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1779" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="C1779" s="9"/>
+      <c r="D1779" s="10" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="1780" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1780" s="8"/>
+      <c r="C1780" s="9"/>
+      <c r="D1780" s="10" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="1781" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1781" s="8"/>
+      <c r="C1781" s="9"/>
+      <c r="D1781" s="10" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="1782" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1782" s="8"/>
+      <c r="C1782" s="9"/>
+      <c r="D1782" s="10" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="1783" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1783" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="C1783" s="9"/>
+      <c r="D1783" s="10"/>
+    </row>
+    <row r="1784" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1784" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="C1784" s="9"/>
+      <c r="D1784" s="10"/>
+    </row>
+    <row r="1785" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1785" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="C1785" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="D1785" s="10" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="1786" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1786" s="16">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="C1786" s="17"/>
+      <c r="D1786" s="24"/>
+    </row>
+    <row r="1787" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1787" s="16">
+        <v>5.2</v>
+      </c>
+      <c r="C1787" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="D1787" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="1788" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1788" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="C1788" s="9"/>
+      <c r="D1788" s="29" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="1789" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1789" s="8"/>
+      <c r="C1789" s="9"/>
+      <c r="D1789" s="29"/>
+    </row>
+    <row r="1790" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1790" s="8"/>
+      <c r="C1790" s="9"/>
+      <c r="D1790" s="29"/>
+    </row>
+    <row r="1791" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1791" s="8">
+        <v>6.2</v>
+      </c>
+      <c r="C1791" s="9"/>
+      <c r="D1791" s="10" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="1792" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1792" s="16">
+        <v>7.1</v>
+      </c>
+      <c r="C1792" s="17"/>
+      <c r="D1792" s="24"/>
+    </row>
+    <row r="1793" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1793" s="16">
+        <v>7.2</v>
+      </c>
+      <c r="C1793" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="D1793" s="24" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1794" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1794" s="8">
+        <v>8.1</v>
+      </c>
+      <c r="C1794" s="9"/>
+      <c r="D1794" s="10"/>
+    </row>
+    <row r="1795" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1795" s="19">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="C1795" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="D1795" s="10" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="1796" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1796" s="8">
+        <v>9.1</v>
+      </c>
+      <c r="C1796" s="9"/>
+      <c r="D1796" s="10"/>
+    </row>
+    <row r="1797" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1797" s="8">
+        <v>9.1999999999999993</v>
+      </c>
+      <c r="C1797" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="D1797" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1798" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1798" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1798" s="21"/>
+      <c r="D1798" s="23"/>
+    </row>
+    <row r="1830" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1830" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="C1830" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1830" s="3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="1831" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1831" s="4"/>
+      <c r="C1831" s="26" t="s">
+        <v>174</v>
+      </c>
+      <c r="D1831" s="27"/>
+    </row>
+    <row r="1832" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1832" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1832" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1832" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1833" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1833" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1833" s="34" t="s">
+        <v>139</v>
+      </c>
+      <c r="D1833" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1834" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1834" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C1834" s="9"/>
+      <c r="D1834" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1835" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1835" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="C1835" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="D1835" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="1836" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1836" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="C1836" s="9"/>
+      <c r="D1836" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1837" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1837" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C1837" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="D1837" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="1838" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1838" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="C1838" s="9"/>
+      <c r="D1838" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1839" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1839" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="C1839" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="D1839" s="10" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="1840" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1840" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="C1840" s="9"/>
+      <c r="D1840" s="10" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="1841" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1841" s="8"/>
+      <c r="C1841" s="9"/>
+      <c r="D1841" s="10" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="1842" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1842" s="8"/>
+      <c r="C1842" s="9"/>
+      <c r="D1842" s="10" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="1843" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1843" s="8"/>
+      <c r="C1843" s="9"/>
+      <c r="D1843" s="10" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="1844" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1844" s="19">
+        <v>4.2</v>
+      </c>
+      <c r="C1844" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="D1844" s="10" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="1845" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1845" s="16">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="C1845" s="17"/>
+      <c r="D1845" s="24"/>
+    </row>
+    <row r="1846" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1846" s="25">
+        <v>5.2</v>
+      </c>
+      <c r="C1846" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="D1846" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="1847" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1847" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="C1847" s="9"/>
+      <c r="D1847" s="29" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="1848" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1848" s="8"/>
+      <c r="C1848" s="9"/>
+      <c r="D1848" s="29"/>
+    </row>
+    <row r="1849" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1849" s="8">
+        <v>6.2</v>
+      </c>
+      <c r="C1849" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="D1849" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1850" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1850" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1850" s="21"/>
+      <c r="D1850" s="23"/>
+    </row>
+    <row r="1889" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1889" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="C1889" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1889" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1890" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1890" s="4"/>
+      <c r="C1890" s="26" t="s">
+        <v>176</v>
+      </c>
+      <c r="D1890" s="27"/>
+    </row>
+    <row r="1891" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1891" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1891" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1891" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1892" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1892" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1892" s="34" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1892" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1893" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1893" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C1893" s="9"/>
+      <c r="D1893" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1894" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1894" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="C1894" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1894" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="1895" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1895" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="C1895" s="9"/>
+      <c r="D1895" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1896" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1896" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C1896" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1896" s="10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="1897" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1897" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="C1897" s="9"/>
+      <c r="D1897" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1898" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1898" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="C1898" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1898" s="10" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="1899" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1899" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="C1899" s="9"/>
+      <c r="D1899" s="10" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="1900" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1900" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="C1900" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="D1900" s="10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="1901" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1901" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="C1901" s="9"/>
+      <c r="D1901" s="10"/>
+    </row>
+    <row r="1902" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1902" s="19">
+        <v>5.2</v>
+      </c>
+      <c r="C1902" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="D1902" s="10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="1903" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1903" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="C1903" s="9"/>
+      <c r="D1903" s="10" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="1904" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1904" s="8">
+        <v>6.2</v>
+      </c>
+      <c r="C1904" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1904" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1905" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1905" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1905" s="21"/>
+      <c r="D1905" s="23"/>
+    </row>
+    <row r="1948" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1948" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="C1948" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1948" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="1949" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1949" s="4"/>
+      <c r="C1949" s="30" t="s">
+        <v>55</v>
+      </c>
+      <c r="D1949" s="31"/>
+    </row>
+    <row r="1950" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1950" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1950" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1950" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1951" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1951" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1951" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1951" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1952" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1952" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C1952" s="9"/>
+      <c r="D1952" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1953" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1953" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="C1953" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="D1953" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="1954" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1954" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="C1954" s="9"/>
+      <c r="D1954" s="10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="1955" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1955" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C1955" s="9"/>
+      <c r="D1955" s="10" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="1956" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1956" s="16">
+        <v>3.1</v>
+      </c>
+      <c r="C1956" s="17"/>
+      <c r="D1956" s="24" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="1957" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1957" s="16">
+        <v>3.2</v>
+      </c>
+      <c r="C1957" s="17"/>
+      <c r="D1957" s="24"/>
+    </row>
+    <row r="1958" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1958" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="C1958" s="9"/>
+      <c r="D1958" s="15"/>
+    </row>
+    <row r="1959" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1959" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="C1959" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1959" s="15" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="1960" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1960" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="C1960" s="9"/>
+      <c r="D1960" s="15"/>
+    </row>
+    <row r="1961" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1961" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="C1961" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D1961" s="15" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="1962" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1962" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="C1962" s="9"/>
+      <c r="D1962" s="15"/>
+    </row>
+    <row r="1963" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1963" s="19">
+        <v>6.2</v>
+      </c>
+      <c r="C1963" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="D1963" s="15" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="1964" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1964" s="16">
+        <v>7.1</v>
+      </c>
+      <c r="C1964" s="17"/>
+      <c r="D1964" s="18"/>
+    </row>
+    <row r="1965" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1965" s="25">
+        <v>7.2</v>
+      </c>
+      <c r="C1965" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="D1965" s="18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="1966" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1966" s="8">
+        <v>8.1</v>
+      </c>
+      <c r="C1966" s="9"/>
+      <c r="D1966" s="29" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="1967" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1967" s="8"/>
+      <c r="C1967" s="9"/>
+      <c r="D1967" s="29"/>
+    </row>
+    <row r="1968" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1968" s="8">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="C1968" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="D1968" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1969" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1969" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1969" s="21"/>
+      <c r="D1969" s="23"/>
+    </row>
+    <row r="2007" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2007" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="C2007" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2007" s="3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="2008" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2008" s="4"/>
+      <c r="C2008" s="30" t="s">
+        <v>183</v>
+      </c>
+      <c r="D2008" s="31"/>
+    </row>
+    <row r="2009" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2009" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2009" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2009" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2010" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2010" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2010" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2010" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2011" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2011" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C2011" s="9"/>
+      <c r="D2011" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2012" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2012" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="C2012" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2012" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2013" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2013" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="C2013" s="9"/>
+      <c r="D2013" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2014" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2014" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C2014" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2014" s="10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2015" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2015" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="C2015" s="9"/>
+      <c r="D2015" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2016" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2016" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="C2016" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="D2016" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2017" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2017" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="C2017" s="9"/>
+      <c r="D2017" s="15"/>
+    </row>
+    <row r="2018" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2018" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="C2018" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="D2018" s="15" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="2019" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2019" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="C2019" s="9"/>
+      <c r="D2019" s="15"/>
+    </row>
+    <row r="2020" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2020" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="C2020" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2020" s="15" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="2021" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2021" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="C2021" s="9"/>
+      <c r="D2021" s="15"/>
+    </row>
+    <row r="2022" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2022" s="8">
+        <v>6.2</v>
+      </c>
+      <c r="C2022" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="D2022" s="15" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2023" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2023" s="8">
+        <v>7.1</v>
+      </c>
+      <c r="C2023" s="9"/>
+      <c r="D2023" s="15"/>
+    </row>
+    <row r="2024" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2024" s="19">
+        <v>7.2</v>
+      </c>
+      <c r="C2024" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="D2024" s="15" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2025" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2025" s="8">
+        <v>8.1</v>
+      </c>
+      <c r="C2025" s="9"/>
+      <c r="D2025" s="10" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="2026" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2026" s="8">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="C2026" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2026" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2027" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2027" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2027" s="21"/>
+      <c r="D2027" s="23"/>
+    </row>
+    <row r="2066" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2066" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="C2066" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2066" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2067" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2067" s="4"/>
+      <c r="C2067" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="D2067" s="27"/>
+    </row>
+    <row r="2068" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2068" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2068" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2068" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2069" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2069" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2069" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2069" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2070" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2070" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C2070" s="9"/>
+      <c r="D2070" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2071" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2071" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="C2071" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="D2071" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2072" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2072" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="C2072" s="9"/>
+      <c r="D2072" s="10" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="2073" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2073" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C2073" s="9"/>
+      <c r="D2073" s="10"/>
+    </row>
+    <row r="2074" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2074" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="C2074" s="9"/>
+      <c r="D2074" s="10"/>
+    </row>
+    <row r="2075" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2075" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="C2075" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2075" s="10" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2076" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2076" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="C2076" s="9"/>
+      <c r="D2076" s="15"/>
+    </row>
+    <row r="2077" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2077" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="C2077" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2077" s="15" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2078" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2078" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="C2078" s="9"/>
+      <c r="D2078" s="29" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="2079" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2079" s="8"/>
+      <c r="C2079" s="9"/>
+      <c r="D2079" s="29"/>
+    </row>
+    <row r="2080" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2080" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="C2080" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="D2080" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2081" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2081" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2081" s="21"/>
+      <c r="D2081" s="23"/>
+    </row>
+    <row r="2125" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2125" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="C2125" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2125" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2126" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2126" s="4"/>
+      <c r="C2126" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="D2126" s="6"/>
+    </row>
+    <row r="2127" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2127" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2127" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2127" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2128" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2128" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2128" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2128" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2129" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2129" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C2129" s="9"/>
+      <c r="D2129" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2130" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2130" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="C2130" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2130" s="10" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="2131" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2131" s="16">
+        <v>2.1</v>
+      </c>
+      <c r="C2131" s="17"/>
+      <c r="D2131" s="24" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2132" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2132" s="16">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C2132" s="17"/>
+      <c r="D2132" s="24"/>
+    </row>
+    <row r="2133" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2133" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="C2133" s="9"/>
+      <c r="D2133" s="15" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="2134" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2134" s="19">
+        <v>3.2</v>
+      </c>
+      <c r="C2134" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2134" s="10" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2135" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2135" s="16">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="C2135" s="17"/>
+      <c r="D2135" s="18"/>
+    </row>
+    <row r="2136" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2136" s="25">
+        <v>4.2</v>
+      </c>
+      <c r="C2136" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2136" s="18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2137" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2137" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="C2137" s="9"/>
+      <c r="D2137" s="29" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="2138" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2138" s="8"/>
+      <c r="C2138" s="9"/>
+      <c r="D2138" s="29"/>
+    </row>
+    <row r="2139" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2139" s="8"/>
+      <c r="C2139" s="9"/>
+      <c r="D2139" s="29"/>
+    </row>
+    <row r="2140" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2140" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="C2140" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2140" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2141" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2141" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2141" s="21"/>
+      <c r="D2141" s="23"/>
+    </row>
+    <row r="2184" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2184" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C2184" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2184" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2185" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2185" s="4"/>
+      <c r="C2185" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="D2185" s="6"/>
+    </row>
+    <row r="2186" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2186" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2186" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2186" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2187" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2187" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2187" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2187" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2188" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2188" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C2188" s="9"/>
+      <c r="D2188" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2189" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2189" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="C2189" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2189" s="10" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="2190" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2190" s="16">
+        <v>2.1</v>
+      </c>
+      <c r="C2190" s="17"/>
+      <c r="D2190" s="24" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2191" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2191" s="16">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C2191" s="17"/>
+      <c r="D2191" s="24"/>
+    </row>
+    <row r="2192" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2192" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="C2192" s="9"/>
+      <c r="D2192" s="15" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="2193" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2193" s="19">
+        <v>3.2</v>
+      </c>
+      <c r="C2193" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2193" s="10" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2194" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2194" s="16">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="C2194" s="17"/>
+      <c r="D2194" s="18"/>
+    </row>
+    <row r="2195" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2195" s="25">
+        <v>4.2</v>
+      </c>
+      <c r="C2195" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2195" s="18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2196" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2196" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="C2196" s="9"/>
+      <c r="D2196" s="29" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="2197" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2197" s="8"/>
+      <c r="C2197" s="9"/>
+      <c r="D2197" s="29"/>
+    </row>
+    <row r="2198" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2198" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="C2198" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2198" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2199" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2199" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2199" s="21"/>
+      <c r="D2199" s="23"/>
+    </row>
   </sheetData>
-  <mergeCells count="33">
+  <mergeCells count="46">
+    <mergeCell ref="D2137:D2139"/>
+    <mergeCell ref="D2196:D2197"/>
+    <mergeCell ref="D1966:D1967"/>
+    <mergeCell ref="C2008:D2008"/>
+    <mergeCell ref="D2078:D2079"/>
+    <mergeCell ref="D1847:D1848"/>
+    <mergeCell ref="C1949:D1949"/>
+    <mergeCell ref="D1730:D1731"/>
+    <mergeCell ref="D1788:D1790"/>
+    <mergeCell ref="C1772:D1772"/>
+    <mergeCell ref="D1541:D1542"/>
+    <mergeCell ref="C1654:D1654"/>
+    <mergeCell ref="D1665:D1666"/>
     <mergeCell ref="C1477:D1477"/>
     <mergeCell ref="D1494:D1495"/>
     <mergeCell ref="D1313:D1315"/>

</xml_diff>

<commit_message>
Added instructions up to 28, added Emulation-Mode document.
</commit_message>
<xml_diff>
--- a/Research/Instructions/Instructions Native SNES.xlsx
+++ b/Research/Instructions/Instructions Native SNES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Projects\BirdSNES\Research\Instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4DB7F92-D5D9-4ED5-8638-5F18291E6BE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68C062E5-22EC-4D06-9456-31DC11DB0E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$D$2220</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$D$2360</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="995" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1052" uniqueCount="193">
   <si>
     <t>BRK (00)</t>
   </si>
@@ -3587,8 +3587,284 @@
     </r>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Discard, then schedule </t>
+    <t>AND (21)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Perform </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &amp;= Operand. If </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>M</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag is set, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L &amp; $80) and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L, otherwise set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.H &amp; $80) and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>JSL (22)</t>
+  </si>
+  <si>
+    <t>Absolute Long</t>
+  </si>
+  <si>
+    <r>
+      <t>Read (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>+0)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Write to (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>-2)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Inc </t>
     </r>
     <r>
       <rPr>
@@ -3609,15 +3885,123 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> -= 1.</t>
-    </r>
-  </si>
-  <si>
-    <t>AND (21)</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Perform </t>
+      <t xml:space="preserve">. Dec. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> by 3.  Copy Address to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Copy Bank to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PB</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>AND (23)</t>
+  </si>
+  <si>
+    <t>BIT (24)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">If </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>M</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag is set, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
     </r>
     <r>
       <rPr>
@@ -3638,7 +4022,144 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> &amp;= Operand. If </t>
+      <t xml:space="preserve">.L &amp; Operand.L), set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (Operand.L &amp; $80), and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>V</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (Operand.L &amp; $40), otherwise set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &amp; Operand), set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (Operand.H &amp; $80), set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>V</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (Operand.H &amp; $40).</t>
+    </r>
+  </si>
+  <si>
+    <t>AND (25)</t>
+  </si>
+  <si>
+    <t>ROL (26)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">If </t>
     </r>
     <r>
       <rPr>
@@ -3670,6 +4191,48 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (Operand.L &amp; $80), perform Operand.L = (Operand.L &lt;&lt; 1) | </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>N</t>
     </r>
     <r>
@@ -3680,28 +4243,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> based off (</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>A</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">.L &amp; $80) and </t>
+      <t xml:space="preserve"> based off (Operand.L &amp; $80) and </t>
     </r>
     <r>
       <rPr>
@@ -3722,28 +4264,49 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> based off </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>A</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">.L, otherwise set </t>
+      <t xml:space="preserve"> based off Operand.L, otherwise set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (Operand.H &amp; $80), perform Operand = (Operand &lt;&lt; 1) | </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, and set </t>
     </r>
     <r>
       <rPr>
@@ -3764,28 +4327,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> based off (</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>A</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">.H &amp; $80) and </t>
+      <t xml:space="preserve"> based off (Operand.H &amp; $80) and </t>
     </r>
     <r>
       <rPr>
@@ -3806,379 +4348,11 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> based off </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>A</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
-    <t>JSL (22)</t>
-  </si>
-  <si>
-    <t>Absolute Long</t>
-  </si>
-  <si>
-    <r>
-      <t>Read (</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>S</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>+0)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Write to (</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>S</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>-2)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Inc </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>PC</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. Dec. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>S</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> by 3.  Copy Address to </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>PC</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. Copy Bank to </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>PB</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
-    <t>AND (23)</t>
-  </si>
-  <si>
-    <t>BIT (24)</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">If </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>M</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> flag is set, set </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Z</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> based off (</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>A</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">.L &amp; Operand.L), set </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>N</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> based off (Operand.L &amp; $80), and set </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>V</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> based off (Operand.L &amp; $40), otherwise set </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Z</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> based off (</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>A</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> &amp; Operand), set </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>N</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> based off (Operand.H &amp; $80), set </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>V</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> based off (Operand.H &amp; $40).</t>
-    </r>
-  </si>
-  <si>
-    <t>AND (25)</t>
+      <t xml:space="preserve"> based off Operand.</t>
+    </r>
+  </si>
+  <si>
+    <t>AND (27)</t>
   </si>
 </sst>
 </file>
@@ -4782,7 +4956,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{236A51FB-68FA-4644-A8C6-D47AA32EBCC5}">
-  <dimension ref="A1:D2199"/>
+  <dimension ref="A1:D2323"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.7109375" customWidth="1"/>
@@ -10467,7 +10641,7 @@
         <v>93</v>
       </c>
       <c r="D1898" s="10" t="s">
-        <v>179</v>
+        <v>97</v>
       </c>
     </row>
     <row r="1899" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -10537,7 +10711,7 @@
     </row>
     <row r="1948" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1948" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C1948" s="2" t="s">
         <v>6</v>
@@ -10707,7 +10881,7 @@
       </c>
       <c r="C1966" s="9"/>
       <c r="D1966" s="29" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="1967" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -10735,7 +10909,7 @@
     </row>
     <row r="2007" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2007" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C2007" s="2" t="s">
         <v>14</v>
@@ -10747,7 +10921,7 @@
     <row r="2008" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2008" s="4"/>
       <c r="C2008" s="30" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D2008" s="31"/>
     </row>
@@ -10845,7 +11019,7 @@
         <v>4.2</v>
       </c>
       <c r="C2018" s="9" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D2018" s="15" t="s">
         <v>97</v>
@@ -10899,7 +11073,7 @@
         <v>7.2</v>
       </c>
       <c r="C2024" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D2024" s="15" t="s">
         <v>36</v>
@@ -10911,7 +11085,7 @@
       </c>
       <c r="C2025" s="9"/>
       <c r="D2025" s="10" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="2026" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -10934,7 +11108,7 @@
     </row>
     <row r="2066" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2066" s="1" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C2066" s="2" t="s">
         <v>24</v>
@@ -11016,7 +11190,7 @@
       <c r="D2074" s="10"/>
     </row>
     <row r="2075" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2075" s="8">
+      <c r="B2075" s="19">
         <v>3.2</v>
       </c>
       <c r="C2075" s="9" t="s">
@@ -11027,20 +11201,20 @@
       </c>
     </row>
     <row r="2076" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2076" s="8">
+      <c r="B2076" s="16">
         <v>4.0999999999999996</v>
       </c>
-      <c r="C2076" s="9"/>
-      <c r="D2076" s="15"/>
+      <c r="C2076" s="17"/>
+      <c r="D2076" s="18"/>
     </row>
     <row r="2077" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2077" s="8">
+      <c r="B2077" s="25">
         <v>4.2</v>
       </c>
-      <c r="C2077" s="9" t="s">
+      <c r="C2077" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="D2077" s="15" t="s">
+      <c r="D2077" s="18" t="s">
         <v>45</v>
       </c>
     </row>
@@ -11050,7 +11224,7 @@
       </c>
       <c r="C2078" s="9"/>
       <c r="D2078" s="29" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="2079" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -11078,7 +11252,7 @@
     </row>
     <row r="2125" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2125" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C2125" s="2" t="s">
         <v>15</v>
@@ -11196,7 +11370,7 @@
       </c>
       <c r="C2137" s="9"/>
       <c r="D2137" s="29" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="2138" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -11229,7 +11403,7 @@
     </row>
     <row r="2184" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2184" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C2184" s="2" t="s">
         <v>15</v>
@@ -11347,7 +11521,7 @@
       </c>
       <c r="C2196" s="9"/>
       <c r="D2196" s="29" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="2197" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -11373,10 +11547,416 @@
       <c r="C2199" s="21"/>
       <c r="D2199" s="23"/>
     </row>
+    <row r="2243" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2243" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C2243" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2243" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2244" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2244" s="4"/>
+      <c r="C2244" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="D2244" s="31"/>
+    </row>
+    <row r="2245" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2245" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2245" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2245" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2246" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2246" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2246" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2246" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2247" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2247" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C2247" s="9"/>
+      <c r="D2247" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2248" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2248" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="C2248" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2248" s="10" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="2249" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2249" s="16">
+        <v>2.1</v>
+      </c>
+      <c r="C2249" s="17"/>
+      <c r="D2249" s="24" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2250" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2250" s="16">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C2250" s="17"/>
+      <c r="D2250" s="24"/>
+    </row>
+    <row r="2251" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2251" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="C2251" s="9"/>
+      <c r="D2251" s="10" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="2252" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2252" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="C2252" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2252" s="10" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2253" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2253" s="16">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="C2253" s="17"/>
+      <c r="D2253" s="18"/>
+    </row>
+    <row r="2254" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2254" s="16">
+        <v>4.2</v>
+      </c>
+      <c r="C2254" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2254" s="18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2255" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2255" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="C2255" s="9"/>
+      <c r="D2255" s="29" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="2256" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2256" s="8"/>
+      <c r="C2256" s="9"/>
+      <c r="D2256" s="29"/>
+    </row>
+    <row r="2257" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2257" s="8"/>
+      <c r="C2257" s="9"/>
+      <c r="D2257" s="29"/>
+    </row>
+    <row r="2258" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2258" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="C2258" s="9"/>
+      <c r="D2258" s="15" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2259" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2259" s="16">
+        <v>6.1</v>
+      </c>
+      <c r="C2259" s="17"/>
+      <c r="D2259" s="18"/>
+    </row>
+    <row r="2260" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2260" s="16">
+        <v>6.2</v>
+      </c>
+      <c r="C2260" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2260" s="18" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2261" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2261" s="8">
+        <v>7.1</v>
+      </c>
+      <c r="C2261" s="9"/>
+      <c r="D2261" s="15"/>
+    </row>
+    <row r="2262" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2262" s="19">
+        <v>7.2</v>
+      </c>
+      <c r="C2262" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="D2262" s="15" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2263" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2263" s="8">
+        <v>8.1</v>
+      </c>
+      <c r="C2263" s="9"/>
+      <c r="D2263" s="10"/>
+    </row>
+    <row r="2264" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2264" s="8">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="C2264" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2264" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2265" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2265" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2265" s="21"/>
+      <c r="D2265" s="23"/>
+    </row>
+    <row r="2302" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2302" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="C2302" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2302" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2303" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2303" s="4"/>
+      <c r="C2303" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="D2303" s="27"/>
+    </row>
+    <row r="2304" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2304" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2304" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2304" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2305" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2305" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2305" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2305" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2306" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2306" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C2306" s="9"/>
+      <c r="D2306" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2307" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2307" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="C2307" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2307" s="10" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="2308" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2308" s="16">
+        <v>2.1</v>
+      </c>
+      <c r="C2308" s="17"/>
+      <c r="D2308" s="24" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2309" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2309" s="16">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C2309" s="17"/>
+      <c r="D2309" s="24"/>
+    </row>
+    <row r="2310" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2310" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="C2310" s="9"/>
+      <c r="D2310" s="10" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="2311" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2311" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="C2311" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2311" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2312" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2312" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="C2312" s="9"/>
+      <c r="D2312" s="15"/>
+    </row>
+    <row r="2313" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2313" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="C2313" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2313" s="15" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2314" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2314" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="C2314" s="9"/>
+      <c r="D2314" s="10"/>
+    </row>
+    <row r="2315" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2315" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="C2315" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="D2315" s="10" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2316" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2316" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="C2316" s="9"/>
+      <c r="D2316" s="10"/>
+    </row>
+    <row r="2317" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2317" s="19">
+        <v>6.2</v>
+      </c>
+      <c r="C2317" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="D2317" s="10" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2318" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2318" s="16">
+        <v>7.1</v>
+      </c>
+      <c r="C2318" s="17"/>
+      <c r="D2318" s="18"/>
+    </row>
+    <row r="2319" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2319" s="25">
+        <v>7.2</v>
+      </c>
+      <c r="C2319" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="D2319" s="18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2320" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2320" s="8">
+        <v>8.1</v>
+      </c>
+      <c r="C2320" s="9"/>
+      <c r="D2320" s="29" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="2321" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2321" s="8"/>
+      <c r="C2321" s="9"/>
+      <c r="D2321" s="29"/>
+    </row>
+    <row r="2322" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2322" s="8">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="C2322" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2322" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2323" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2323" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2323" s="21"/>
+      <c r="D2323" s="23"/>
+    </row>
   </sheetData>
-  <mergeCells count="46">
+  <mergeCells count="49">
+    <mergeCell ref="D2320:D2321"/>
+    <mergeCell ref="D2255:D2257"/>
     <mergeCell ref="D2137:D2139"/>
     <mergeCell ref="D2196:D2197"/>
+    <mergeCell ref="C2244:D2244"/>
     <mergeCell ref="D1966:D1967"/>
     <mergeCell ref="C2008:D2008"/>
     <mergeCell ref="D2078:D2079"/>

</xml_diff>

<commit_message>
Instructions up to 43.
</commit_message>
<xml_diff>
--- a/Research/Instructions/Instructions Native SNES.xlsx
+++ b/Research/Instructions/Instructions Native SNES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Projects\BirdSNES\Research\Instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67F1A26A-AFCD-4C0A-B359-3E10435ED757}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8DCFD44-5E45-4EB3-96CB-AC7581C4D15A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$3776</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$4012</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1646" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1738" uniqueCount="243">
   <si>
     <t>BRK (00)</t>
   </si>
@@ -6197,6 +6197,487 @@
   </si>
   <si>
     <t>AND (3F)</t>
+  </si>
+  <si>
+    <t>Direct, X (Read/Modify/Write)</t>
+  </si>
+  <si>
+    <t>RTI (40)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>P</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to Operand.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Store as </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PB</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Read (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>+3)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Inc. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> by 3. Set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PB</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to Bank. Set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to Operand. If </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag is set, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L.</t>
+    </r>
+  </si>
+  <si>
+    <t>EOR (41)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Perform </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ^= Operand. If </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>M</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag is set, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L &amp; $80) and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L, otherwise set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.H &amp; $80) and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>WDM (42)</t>
+  </si>
+  <si>
+    <t>EOR (43)</t>
   </si>
 </sst>
 </file>
@@ -6801,7 +7282,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{236A51FB-68FA-4644-A8C6-D47AA32EBCC5}">
-  <dimension ref="A1:C3737"/>
+  <dimension ref="A1:C3969"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25.7109375" customWidth="1"/>
@@ -10656,7 +11137,7 @@
     <row r="1300" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1300" s="4"/>
       <c r="B1300" s="31" t="s">
-        <v>142</v>
+        <v>233</v>
       </c>
       <c r="C1300" s="32"/>
     </row>
@@ -17647,8 +18128,614 @@
       <c r="B3737" s="21"/>
       <c r="C3737" s="23"/>
     </row>
+    <row r="3777" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3777" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="B3777" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C3777" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3778" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3778" s="4"/>
+      <c r="B3778" s="26" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3778" s="27"/>
+    </row>
+    <row r="3779" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3779" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3779" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3779" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3780" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3780" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3780" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3780" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3781" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3781" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B3781" s="9"/>
+      <c r="C3781" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3782" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3782" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B3782" s="9"/>
+      <c r="C3782" s="10"/>
+    </row>
+    <row r="3783" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3783" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B3783" s="9"/>
+      <c r="C3783" s="10"/>
+    </row>
+    <row r="3784" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3784" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B3784" s="9"/>
+      <c r="C3784" s="10"/>
+    </row>
+    <row r="3785" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3785" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B3785" s="9"/>
+      <c r="C3785" s="15" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="3786" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3786" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B3786" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="C3786" s="10" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="3787" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3787" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B3787" s="9"/>
+      <c r="C3787" s="15" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="3788" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3788" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B3788" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="C3788" s="15" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="3789" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3789" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B3789" s="9"/>
+      <c r="C3789" s="10"/>
+    </row>
+    <row r="3790" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3790" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="B3790" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="C3790" s="10" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3791" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3791" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="B3791" s="9"/>
+      <c r="C3791" s="10"/>
+    </row>
+    <row r="3792" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3792" s="19">
+        <v>6.2</v>
+      </c>
+      <c r="B3792" s="9" t="s">
+        <v>237</v>
+      </c>
+      <c r="C3792" s="10" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="3793" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3793" s="8">
+        <v>7.1</v>
+      </c>
+      <c r="B3793" s="9"/>
+      <c r="C3793" s="10" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="3794" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3794" s="8">
+        <v>7.2</v>
+      </c>
+      <c r="B3794" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3794" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3795" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3795" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3795" s="21"/>
+      <c r="C3795" s="23"/>
+    </row>
+    <row r="3836" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3836" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="B3836" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3836" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3837" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3837" s="4"/>
+      <c r="B3837" s="31" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3837" s="32"/>
+    </row>
+    <row r="3838" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3838" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3838" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3838" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3839" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3839" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3839" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3839" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3840" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3840" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B3840" s="9"/>
+      <c r="C3840" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3841" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3841" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B3841" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="C3841" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3842" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3842" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B3842" s="9"/>
+      <c r="C3842" s="10" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3843" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3843" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B3843" s="9"/>
+      <c r="C3843" s="10" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="3844" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3844" s="16">
+        <v>3.1</v>
+      </c>
+      <c r="B3844" s="17"/>
+      <c r="C3844" s="18" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3845" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3845" s="16">
+        <v>3.2</v>
+      </c>
+      <c r="B3845" s="17"/>
+      <c r="C3845" s="24"/>
+    </row>
+    <row r="3846" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3846" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B3846" s="9"/>
+      <c r="C3846" s="15"/>
+    </row>
+    <row r="3847" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3847" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B3847" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3847" s="15" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3848" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3848" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B3848" s="9"/>
+      <c r="C3848" s="15"/>
+    </row>
+    <row r="3849" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3849" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="B3849" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3849" s="15" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3850" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3850" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="B3850" s="9"/>
+      <c r="C3850" s="10"/>
+    </row>
+    <row r="3851" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3851" s="19">
+        <v>6.2</v>
+      </c>
+      <c r="B3851" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C3851" s="10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3852" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3852" s="16">
+        <v>7.1</v>
+      </c>
+      <c r="B3852" s="17"/>
+      <c r="C3852" s="24"/>
+    </row>
+    <row r="3853" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3853" s="25">
+        <v>7.2</v>
+      </c>
+      <c r="B3853" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="C3853" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3854" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3854" s="8">
+        <v>8.1</v>
+      </c>
+      <c r="B3854" s="9"/>
+      <c r="C3854" s="30" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="3855" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3855" s="8"/>
+      <c r="B3855" s="9"/>
+      <c r="C3855" s="30"/>
+    </row>
+    <row r="3856" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3856" s="8">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="B3856" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3856" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3857" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3857" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3857" s="21"/>
+      <c r="C3857" s="23"/>
+    </row>
+    <row r="3895" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3895" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="B3895" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3895" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3896" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3896" s="4"/>
+      <c r="B3896" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3896" s="27"/>
+    </row>
+    <row r="3897" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3897" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3897" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3897" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3898" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3898" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3898" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3898" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3899" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3899" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B3899" s="9"/>
+      <c r="C3899" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3900" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3900" s="19">
+        <v>1.2</v>
+      </c>
+      <c r="B3900" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3900" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3901" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3901" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B3901" s="9"/>
+      <c r="C3901" s="10" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3902" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3902" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B3902" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3902" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3903" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3903" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3903" s="21"/>
+      <c r="C3903" s="23"/>
+    </row>
+    <row r="3954" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3954" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="B3954" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3954" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3955" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3955" s="4"/>
+      <c r="B3955" s="31" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3955" s="32"/>
+    </row>
+    <row r="3956" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3956" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3956" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3956" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3957" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3957" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3957" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3957" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3958" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3958" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B3958" s="9"/>
+      <c r="C3958" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3959" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3959" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B3959" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3959" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3960" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3960" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B3960" s="9"/>
+      <c r="C3960" s="10" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="3961" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3961" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B3961" s="9"/>
+      <c r="C3961" s="10"/>
+    </row>
+    <row r="3962" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3962" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B3962" s="9"/>
+      <c r="C3962" s="15"/>
+    </row>
+    <row r="3963" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3963" s="19">
+        <v>3.2</v>
+      </c>
+      <c r="B3963" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3963" s="10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3964" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3964" s="16">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B3964" s="17"/>
+      <c r="C3964" s="18"/>
+    </row>
+    <row r="3965" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3965" s="25">
+        <v>4.2</v>
+      </c>
+      <c r="B3965" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3965" s="18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3966" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3966" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B3966" s="9"/>
+      <c r="C3966" s="30" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="3967" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3967" s="8"/>
+      <c r="B3967" s="9"/>
+      <c r="C3967" s="30"/>
+    </row>
+    <row r="3968" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3968" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="B3968" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3968" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3969" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3969" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3969" s="21"/>
+      <c r="C3969" s="23"/>
+    </row>
   </sheetData>
-  <mergeCells count="78">
+  <mergeCells count="82">
+    <mergeCell ref="B3955:C3955"/>
+    <mergeCell ref="C3966:C3967"/>
+    <mergeCell ref="C3854:C3855"/>
+    <mergeCell ref="B3837:C3837"/>
     <mergeCell ref="B3719:C3719"/>
     <mergeCell ref="C3734:C3735"/>
     <mergeCell ref="C3559:C3561"/>
@@ -17730,6 +18817,9 @@
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup scale="79" orientation="portrait" r:id="rId1"/>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="3776" max="2" man="1"/>
+  </rowBreaks>
   <colBreaks count="1" manualBreakCount="1">
     <brk id="4" max="1048575" man="1"/>
   </colBreaks>

</xml_diff>

<commit_message>
Instructions up to B1.
</commit_message>
<xml_diff>
--- a/Research/Instructions/Instructions Native SNES.xlsx
+++ b/Research/Instructions/Instructions Native SNES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Projects\BirdSNES\Research\Instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30663A2D-5CF5-4410-BF9B-CE176A0D7EEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36DB2B1A-1CD9-4765-8CEA-188692191B7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$9437</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$10381</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4436" uniqueCount="455">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4800" uniqueCount="481">
   <si>
     <t>BRK (00)</t>
   </si>
@@ -13158,6 +13158,2225 @@
   </si>
   <si>
     <t>Absolute Long, X (Write)</t>
+  </si>
+  <si>
+    <t>LDY (A0)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Inc. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. If </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag is set, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L to Operand.L, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L &amp; $80), and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L, otherwise set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to Operand, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.H &amp; $80), and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Store as Operand. If </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag is set, skip the next cycle.</t>
+    </r>
+  </si>
+  <si>
+    <t>LDA (A1)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">If </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>M</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag is set, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L to Operand.L, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L &amp; $80), and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L, otherwise set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to Operand, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.H &amp; $80), and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>LDX (A2)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Inc. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. If </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag is set, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L to Operand.L, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L &amp; $80), and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L, otherwise set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to Operand, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.H &amp; $80), and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>LDA (A3)</t>
+  </si>
+  <si>
+    <t>LDY (A4)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">If </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag is set, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L to Operand.L, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L &amp; $80), and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L, otherwise set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to Operand, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.H &amp; $80), and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>LDA (A5)</t>
+  </si>
+  <si>
+    <t>LDX (A6)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">If </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag is set, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L to Operand.L, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L &amp; $80), and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L, otherwise set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to Operand, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.H &amp; $80), and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>LDA (A7)</t>
+  </si>
+  <si>
+    <t>TAY (A8)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">If </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag is set, perform </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L = </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L &amp; $80), and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L, otherwise perform </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> = </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.H &amp; $80), and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>LDA (A9)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Inc. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. If </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>M</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag is set, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L to Operand.L, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L &amp; $80), and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L, otherwise set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to Operand, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.H &amp; $80), and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>TAX (AA)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">If </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag is set, perform </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L = </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L &amp; $80), and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L, otherwise perform </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> = </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.H &amp; $80), and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>PLB (AB)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>DB</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to Bank, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>DB</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &amp; $80), and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>DB</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>LDY (AC)</t>
+  </si>
+  <si>
+    <t>LDA (AD)</t>
+  </si>
+  <si>
+    <t>LDX (AE)</t>
+  </si>
+  <si>
+    <t>LDA (AF)</t>
   </si>
 </sst>
 </file>
@@ -13771,7 +15990,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{236A51FB-68FA-4644-A8C6-D47AA32EBCC5}">
-  <dimension ref="A1:C9398"/>
+  <dimension ref="A1:C10341"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25.7109375" customWidth="1"/>
@@ -43044,12 +45263,2284 @@
       <c r="B9398" s="21"/>
       <c r="C9398" s="22"/>
     </row>
+    <row r="9438" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9438" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="B9438" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9438" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9439" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9439" s="4"/>
+      <c r="B9439" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9439" s="27"/>
+    </row>
+    <row r="9440" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9440" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9440" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9440" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9441" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9441" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9441" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9441" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9442" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9442" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B9442" s="9"/>
+      <c r="C9442" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9443" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9443" s="19">
+        <v>1.2</v>
+      </c>
+      <c r="B9443" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9443" s="10" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="9444" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9444" s="16">
+        <v>2.1</v>
+      </c>
+      <c r="B9444" s="17"/>
+      <c r="C9444" s="24" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9445" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9445" s="25">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B9445" s="31" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9445" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9446" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9446" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B9446" s="9"/>
+      <c r="C9446" s="36" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="9447" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9447" s="8"/>
+      <c r="B9447" s="9"/>
+      <c r="C9447" s="36"/>
+    </row>
+    <row r="9448" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9448" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B9448" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9448" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9449" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9449" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9449" s="21"/>
+      <c r="C9449" s="22"/>
+    </row>
+    <row r="9497" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9497" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="B9497" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9497" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9498" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9498" s="4"/>
+      <c r="B9498" s="34" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9498" s="35"/>
+    </row>
+    <row r="9499" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9499" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9499" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9499" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9500" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9500" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9500" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9500" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9501" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9501" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B9501" s="9"/>
+      <c r="C9501" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9502" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9502" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B9502" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9502" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9503" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9503" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B9503" s="9"/>
+      <c r="C9503" s="10" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="9504" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9504" s="8"/>
+      <c r="B9504" s="9"/>
+      <c r="C9504" s="10" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="9505" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9505" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B9505" s="9"/>
+      <c r="C9505" s="10" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="9506" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9506" s="16">
+        <v>3.1</v>
+      </c>
+      <c r="B9506" s="17"/>
+      <c r="C9506" s="24" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9507" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9507" s="16">
+        <v>3.2</v>
+      </c>
+      <c r="B9507" s="17"/>
+      <c r="C9507" s="24"/>
+    </row>
+    <row r="9508" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9508" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B9508" s="9"/>
+      <c r="C9508" s="10"/>
+    </row>
+    <row r="9509" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9509" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B9509" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9509" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9510" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9510" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B9510" s="9"/>
+      <c r="C9510" s="10"/>
+    </row>
+    <row r="9511" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9511" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="B9511" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9511" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9512" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9512" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="B9512" s="9"/>
+      <c r="C9512" s="10"/>
+    </row>
+    <row r="9513" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9513" s="19">
+        <v>6.2</v>
+      </c>
+      <c r="B9513" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C9513" s="10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9514" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9514" s="16">
+        <v>7.1</v>
+      </c>
+      <c r="B9514" s="17"/>
+      <c r="C9514" s="24"/>
+    </row>
+    <row r="9515" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9515" s="25">
+        <v>7.2</v>
+      </c>
+      <c r="B9515" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="C9515" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9516" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9516" s="8">
+        <v>8.1</v>
+      </c>
+      <c r="B9516" s="32"/>
+      <c r="C9516" s="36" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="9517" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9517" s="8"/>
+      <c r="B9517" s="32"/>
+      <c r="C9517" s="36"/>
+    </row>
+    <row r="9518" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9518" s="8">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="B9518" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9518" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9519" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9519" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9519" s="21"/>
+      <c r="C9519" s="22"/>
+    </row>
+    <row r="9556" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9556" s="1" t="s">
+        <v>460</v>
+      </c>
+      <c r="B9556" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9556" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9557" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9557" s="4"/>
+      <c r="B9557" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9557" s="27"/>
+    </row>
+    <row r="9558" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9558" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9558" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9558" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9559" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9559" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9559" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9559" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9560" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9560" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B9560" s="9"/>
+      <c r="C9560" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9561" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9561" s="19">
+        <v>1.2</v>
+      </c>
+      <c r="B9561" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9561" s="10" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="9562" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9562" s="16">
+        <v>2.1</v>
+      </c>
+      <c r="B9562" s="17"/>
+      <c r="C9562" s="24" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9563" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9563" s="25">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B9563" s="31" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9563" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9564" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9564" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B9564" s="9"/>
+      <c r="C9564" s="36" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="9565" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9565" s="8"/>
+      <c r="B9565" s="9"/>
+      <c r="C9565" s="36"/>
+    </row>
+    <row r="9566" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9566" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B9566" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9566" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9567" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9567" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9567" s="21"/>
+      <c r="C9567" s="22"/>
+    </row>
+    <row r="9615" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9615" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="B9615" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9615" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9616" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9616" s="4"/>
+      <c r="B9616" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="C9616" s="27"/>
+    </row>
+    <row r="9617" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9617" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9617" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9617" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9618" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9618" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9618" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9618" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9619" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9619" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B9619" s="9"/>
+      <c r="C9619" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9620" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9620" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B9620" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9620" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9621" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9621" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B9621" s="9"/>
+      <c r="C9621" s="10" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="9622" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9622" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B9622" s="9"/>
+      <c r="C9622" s="10"/>
+    </row>
+    <row r="9623" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9623" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B9623" s="32"/>
+      <c r="C9623" s="10"/>
+    </row>
+    <row r="9624" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9624" s="19">
+        <v>3.2</v>
+      </c>
+      <c r="B9624" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9624" s="10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9625" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9625" s="16">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B9625" s="31"/>
+      <c r="C9625" s="24"/>
+    </row>
+    <row r="9626" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9626" s="25">
+        <v>4.2</v>
+      </c>
+      <c r="B9626" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9626" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9627" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9627" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B9627" s="9"/>
+      <c r="C9627" s="36" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="9628" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9628" s="8"/>
+      <c r="B9628" s="9"/>
+      <c r="C9628" s="36"/>
+    </row>
+    <row r="9629" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9629" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="B9629" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9629" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9630" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9630" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9630" s="21"/>
+      <c r="C9630" s="22"/>
+    </row>
+    <row r="9674" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9674" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="B9674" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9674" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9675" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9675" s="4"/>
+      <c r="B9675" s="26" t="s">
+        <v>82</v>
+      </c>
+      <c r="C9675" s="27"/>
+    </row>
+    <row r="9676" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9676" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9676" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9676" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9677" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9677" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9677" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9677" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9678" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9678" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B9678" s="9"/>
+      <c r="C9678" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9679" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9679" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B9679" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9679" s="10" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="9680" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9680" s="16">
+        <v>2.1</v>
+      </c>
+      <c r="B9680" s="17"/>
+      <c r="C9680" s="24" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9681" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9681" s="16">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B9681" s="17"/>
+      <c r="C9681" s="24"/>
+    </row>
+    <row r="9682" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9682" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B9682" s="32"/>
+      <c r="C9682" s="10" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="9683" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9683" s="19">
+        <v>3.2</v>
+      </c>
+      <c r="B9683" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9683" s="10" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="9684" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9684" s="16">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B9684" s="31"/>
+      <c r="C9684" s="24"/>
+    </row>
+    <row r="9685" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9685" s="25">
+        <v>4.2</v>
+      </c>
+      <c r="B9685" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9685" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9686" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9686" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B9686" s="9"/>
+      <c r="C9686" s="36" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="9687" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9687" s="8"/>
+      <c r="B9687" s="9"/>
+      <c r="C9687" s="36"/>
+    </row>
+    <row r="9688" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9688" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="B9688" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9688" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9689" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9689" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9689" s="21"/>
+      <c r="C9689" s="22"/>
+    </row>
+    <row r="9733" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9733" s="1" t="s">
+        <v>465</v>
+      </c>
+      <c r="B9733" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9733" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9734" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9734" s="4"/>
+      <c r="B9734" s="26" t="s">
+        <v>82</v>
+      </c>
+      <c r="C9734" s="27"/>
+    </row>
+    <row r="9735" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9735" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9735" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9735" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9736" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9736" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9736" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9736" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9737" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9737" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B9737" s="9"/>
+      <c r="C9737" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9738" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9738" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B9738" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9738" s="10" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="9739" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9739" s="16">
+        <v>2.1</v>
+      </c>
+      <c r="B9739" s="17"/>
+      <c r="C9739" s="24" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9740" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9740" s="16">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B9740" s="17"/>
+      <c r="C9740" s="24"/>
+    </row>
+    <row r="9741" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9741" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B9741" s="32"/>
+      <c r="C9741" s="10" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="9742" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9742" s="19">
+        <v>3.2</v>
+      </c>
+      <c r="B9742" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9742" s="10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9743" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9743" s="16">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B9743" s="31"/>
+      <c r="C9743" s="24"/>
+    </row>
+    <row r="9744" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9744" s="25">
+        <v>4.2</v>
+      </c>
+      <c r="B9744" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9744" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9745" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9745" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B9745" s="9"/>
+      <c r="C9745" s="36" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="9746" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9746" s="8"/>
+      <c r="B9746" s="9"/>
+      <c r="C9746" s="36"/>
+    </row>
+    <row r="9747" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9747" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="B9747" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9747" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9748" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9748" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9748" s="21"/>
+      <c r="C9748" s="22"/>
+    </row>
+    <row r="9792" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9792" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="B9792" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9792" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9793" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9793" s="4"/>
+      <c r="B9793" s="26" t="s">
+        <v>82</v>
+      </c>
+      <c r="C9793" s="27"/>
+    </row>
+    <row r="9794" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9794" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9794" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9794" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9795" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9795" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9795" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9795" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9796" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9796" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B9796" s="9"/>
+      <c r="C9796" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9797" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9797" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B9797" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9797" s="10" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="9798" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9798" s="16">
+        <v>2.1</v>
+      </c>
+      <c r="B9798" s="17"/>
+      <c r="C9798" s="24" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9799" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9799" s="16">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B9799" s="17"/>
+      <c r="C9799" s="24"/>
+    </row>
+    <row r="9800" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9800" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B9800" s="32"/>
+      <c r="C9800" s="10" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="9801" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9801" s="19">
+        <v>3.2</v>
+      </c>
+      <c r="B9801" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9801" s="10" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="9802" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9802" s="16">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B9802" s="31"/>
+      <c r="C9802" s="24"/>
+    </row>
+    <row r="9803" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9803" s="25">
+        <v>4.2</v>
+      </c>
+      <c r="B9803" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9803" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9804" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9804" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B9804" s="9"/>
+      <c r="C9804" s="36" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="9805" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9805" s="8"/>
+      <c r="B9805" s="9"/>
+      <c r="C9805" s="36"/>
+    </row>
+    <row r="9806" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9806" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="B9806" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9806" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9807" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9807" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9807" s="21"/>
+      <c r="C9807" s="22"/>
+    </row>
+    <row r="9851" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9851" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="B9851" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9851" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9852" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9852" s="4"/>
+      <c r="B9852" s="26" t="s">
+        <v>87</v>
+      </c>
+      <c r="C9852" s="27"/>
+    </row>
+    <row r="9853" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9853" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9853" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9853" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9854" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9854" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9854" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9854" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9855" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9855" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B9855" s="9"/>
+      <c r="C9855" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9856" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9856" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B9856" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9856" s="10" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="9857" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9857" s="16">
+        <v>2.1</v>
+      </c>
+      <c r="B9857" s="17"/>
+      <c r="C9857" s="24" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9858" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9858" s="16">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B9858" s="17"/>
+      <c r="C9858" s="24"/>
+    </row>
+    <row r="9859" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9859" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B9859" s="32"/>
+      <c r="C9859" s="10" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="9860" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9860" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B9860" s="32" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9860" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9861" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9861" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B9861" s="32"/>
+      <c r="C9861" s="10"/>
+    </row>
+    <row r="9862" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9862" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B9862" s="32" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9862" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9863" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9863" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B9863" s="32"/>
+      <c r="C9863" s="10"/>
+    </row>
+    <row r="9864" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9864" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="B9864" s="32" t="s">
+        <v>84</v>
+      </c>
+      <c r="C9864" s="10" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="9865" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9865" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="B9865" s="32"/>
+      <c r="C9865" s="10"/>
+    </row>
+    <row r="9866" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9866" s="19">
+        <v>6.2</v>
+      </c>
+      <c r="B9866" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C9866" s="10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9867" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9867" s="16">
+        <v>7.1</v>
+      </c>
+      <c r="B9867" s="31"/>
+      <c r="C9867" s="24"/>
+    </row>
+    <row r="9868" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9868" s="25">
+        <v>7.2</v>
+      </c>
+      <c r="B9868" s="33" t="s">
+        <v>349</v>
+      </c>
+      <c r="C9868" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9869" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9869" s="25"/>
+      <c r="B9869" s="33"/>
+      <c r="C9869" s="24"/>
+    </row>
+    <row r="9870" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9870" s="8">
+        <v>8.1</v>
+      </c>
+      <c r="B9870" s="9"/>
+      <c r="C9870" s="36" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="9871" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9871" s="8"/>
+      <c r="B9871" s="9"/>
+      <c r="C9871" s="36"/>
+    </row>
+    <row r="9872" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9872" s="8">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="B9872" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9872" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9873" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9873" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9873" s="21"/>
+      <c r="C9873" s="22"/>
+    </row>
+    <row r="9910" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9910" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B9910" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9910" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9911" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9911" s="4"/>
+      <c r="B9911" s="26" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9911" s="27"/>
+    </row>
+    <row r="9912" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9912" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9912" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9912" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9913" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9913" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9913" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9913" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9914" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9914" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B9914" s="9"/>
+      <c r="C9914" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9915" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9915" s="19">
+        <v>1.2</v>
+      </c>
+      <c r="B9915" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9915" s="10" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="9916" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9916" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B9916" s="9"/>
+      <c r="C9916" s="36" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="9917" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9917" s="8"/>
+      <c r="B9917" s="9"/>
+      <c r="C9917" s="36"/>
+    </row>
+    <row r="9918" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9918" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B9918" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9918" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9919" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9919" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9919" s="21"/>
+      <c r="C9919" s="22"/>
+    </row>
+    <row r="9969" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9969" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="B9969" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9969" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9970" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9970" s="4"/>
+      <c r="B9970" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9970" s="27"/>
+    </row>
+    <row r="9971" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9971" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9971" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9971" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9972" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9972" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9972" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9972" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9973" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9973" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B9973" s="9"/>
+      <c r="C9973" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9974" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9974" s="19">
+        <v>1.2</v>
+      </c>
+      <c r="B9974" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9974" s="10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9975" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9975" s="16">
+        <v>2.1</v>
+      </c>
+      <c r="B9975" s="17"/>
+      <c r="C9975" s="24" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9976" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9976" s="25">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B9976" s="31" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9976" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9977" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9977" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B9977" s="9"/>
+      <c r="C9977" s="36" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="9978" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9978" s="8"/>
+      <c r="B9978" s="9"/>
+      <c r="C9978" s="36"/>
+    </row>
+    <row r="9979" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9979" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B9979" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9979" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9980" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9980" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9980" s="21"/>
+      <c r="C9980" s="22"/>
+    </row>
+    <row r="10028" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10028" s="1" t="s">
+        <v>473</v>
+      </c>
+      <c r="B10028" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10028" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10029" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10029" s="4"/>
+      <c r="B10029" s="26" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10029" s="27"/>
+    </row>
+    <row r="10030" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10030" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10030" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10030" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10031" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10031" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10031" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10031" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10032" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10032" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B10032" s="9"/>
+      <c r="C10032" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10033" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10033" s="19">
+        <v>1.2</v>
+      </c>
+      <c r="B10033" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10033" s="10" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="10034" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10034" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B10034" s="9"/>
+      <c r="C10034" s="36" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="10035" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10035" s="8"/>
+      <c r="B10035" s="9"/>
+      <c r="C10035" s="36"/>
+    </row>
+    <row r="10036" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10036" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B10036" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10036" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10037" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10037" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10037" s="21"/>
+      <c r="C10037" s="22"/>
+    </row>
+    <row r="10087" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10087" s="1" t="s">
+        <v>475</v>
+      </c>
+      <c r="B10087" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10087" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10088" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10088" s="4"/>
+      <c r="B10088" s="26" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10088" s="27"/>
+    </row>
+    <row r="10089" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10089" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10089" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10089" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10090" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10090" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10090" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="C10090" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10091" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10091" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B10091" s="9"/>
+      <c r="C10091" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10092" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10092" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B10092" s="32"/>
+      <c r="C10092" s="10"/>
+    </row>
+    <row r="10093" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10093" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B10093" s="9"/>
+      <c r="C10093" s="10"/>
+    </row>
+    <row r="10094" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10094" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B10094" s="9"/>
+      <c r="C10094" s="10"/>
+    </row>
+    <row r="10095" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10095" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B10095" s="9"/>
+      <c r="C10095" s="10" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="10096" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10096" s="19">
+        <v>3.2</v>
+      </c>
+      <c r="B10096" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="C10096" s="10" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="10097" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10097" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B10097" s="9"/>
+      <c r="C10097" s="10" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="10098" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10098" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B10098" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10098" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10099" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10099" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10099" s="21"/>
+      <c r="C10099" s="22"/>
+    </row>
+    <row r="10146" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10146" s="1" t="s">
+        <v>477</v>
+      </c>
+      <c r="B10146" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10146" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10147" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10147" s="4"/>
+      <c r="B10147" s="26" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10147" s="27"/>
+    </row>
+    <row r="10148" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10148" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10148" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10148" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10149" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10149" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10149" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10149" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10150" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10150" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B10150" s="9"/>
+      <c r="C10150" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10151" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10151" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B10151" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10151" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10152" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10152" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B10152" s="9"/>
+      <c r="C10152" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10153" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10153" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B10153" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10153" s="10" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="10154" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10154" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B10154" s="9"/>
+      <c r="C10154" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10155" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10155" s="19">
+        <v>3.2</v>
+      </c>
+      <c r="B10155" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="C10155" s="10" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="10156" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10156" s="16">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B10156" s="17"/>
+      <c r="C10156" s="24"/>
+    </row>
+    <row r="10157" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10157" s="25">
+        <v>4.2</v>
+      </c>
+      <c r="B10157" s="31" t="s">
+        <v>103</v>
+      </c>
+      <c r="C10157" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10158" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10158" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B10158" s="9"/>
+      <c r="C10158" s="36" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="10159" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10159" s="8"/>
+      <c r="B10159" s="9"/>
+      <c r="C10159" s="36"/>
+    </row>
+    <row r="10160" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10160" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="B10160" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10160" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10161" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10161" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10161" s="21"/>
+      <c r="C10161" s="22"/>
+    </row>
+    <row r="10205" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10205" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="B10205" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10205" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10206" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10206" s="4"/>
+      <c r="B10206" s="26" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10206" s="27"/>
+    </row>
+    <row r="10207" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10207" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10207" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10207" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10208" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10208" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10208" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10208" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10209" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10209" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B10209" s="9"/>
+      <c r="C10209" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10210" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10210" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B10210" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10210" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10211" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10211" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B10211" s="9"/>
+      <c r="C10211" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10212" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10212" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B10212" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10212" s="10" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="10213" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10213" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B10213" s="9"/>
+      <c r="C10213" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10214" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10214" s="19">
+        <v>3.2</v>
+      </c>
+      <c r="B10214" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="C10214" s="10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10215" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10215" s="16">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B10215" s="17"/>
+      <c r="C10215" s="24"/>
+    </row>
+    <row r="10216" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10216" s="25">
+        <v>4.2</v>
+      </c>
+      <c r="B10216" s="31" t="s">
+        <v>103</v>
+      </c>
+      <c r="C10216" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10217" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10217" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B10217" s="9"/>
+      <c r="C10217" s="36" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="10218" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10218" s="8"/>
+      <c r="B10218" s="9"/>
+      <c r="C10218" s="36"/>
+    </row>
+    <row r="10219" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10219" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="B10219" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10219" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10220" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10220" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10220" s="21"/>
+      <c r="C10220" s="22"/>
+    </row>
+    <row r="10264" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10264" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="B10264" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10264" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10265" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10265" s="4"/>
+      <c r="B10265" s="26" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10265" s="27"/>
+    </row>
+    <row r="10266" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10266" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10266" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10266" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10267" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10267" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10267" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10267" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10268" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10268" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B10268" s="9"/>
+      <c r="C10268" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10269" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10269" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B10269" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10269" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10270" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10270" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B10270" s="9"/>
+      <c r="C10270" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10271" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10271" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B10271" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10271" s="10" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="10272" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10272" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B10272" s="9"/>
+      <c r="C10272" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10273" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10273" s="19">
+        <v>3.2</v>
+      </c>
+      <c r="B10273" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="C10273" s="10" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="10274" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10274" s="16">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B10274" s="17"/>
+      <c r="C10274" s="24"/>
+    </row>
+    <row r="10275" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10275" s="25">
+        <v>4.2</v>
+      </c>
+      <c r="B10275" s="31" t="s">
+        <v>103</v>
+      </c>
+      <c r="C10275" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10276" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10276" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B10276" s="9"/>
+      <c r="C10276" s="36" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="10277" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10277" s="8"/>
+      <c r="B10277" s="9"/>
+      <c r="C10277" s="36"/>
+    </row>
+    <row r="10278" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10278" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="B10278" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10278" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10279" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10279" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10279" s="21"/>
+      <c r="C10279" s="22"/>
+    </row>
+    <row r="10323" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10323" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="B10323" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10323" s="3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="10324" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10324" s="4"/>
+      <c r="B10324" s="26" t="s">
+        <v>111</v>
+      </c>
+      <c r="C10324" s="27"/>
+    </row>
+    <row r="10325" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10325" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10325" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10325" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10326" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10326" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10326" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10326" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10327" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10327" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B10327" s="9"/>
+      <c r="C10327" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10328" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10328" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B10328" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10328" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10329" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10329" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B10329" s="32"/>
+      <c r="C10329" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10330" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10330" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B10330" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10330" s="10" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="10331" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10331" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B10331" s="9"/>
+      <c r="C10331" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10332" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10332" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B10332" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10332" s="10" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="10333" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10333" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B10333" s="9"/>
+      <c r="C10333" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10334" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10334" s="19">
+        <v>4.2</v>
+      </c>
+      <c r="B10334" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="C10334" s="10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10335" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10335" s="16">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B10335" s="17"/>
+      <c r="C10335" s="24"/>
+    </row>
+    <row r="10336" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10336" s="25">
+        <v>5.2</v>
+      </c>
+      <c r="B10336" s="33" t="s">
+        <v>350</v>
+      </c>
+      <c r="C10336" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10337" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10337" s="25"/>
+      <c r="B10337" s="33"/>
+      <c r="C10337" s="24"/>
+    </row>
+    <row r="10338" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10338" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="B10338" s="9"/>
+      <c r="C10338" s="36" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="10339" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10339" s="8"/>
+      <c r="B10339" s="9"/>
+      <c r="C10339" s="36"/>
+    </row>
+    <row r="10340" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10340" s="8">
+        <v>6.2</v>
+      </c>
+      <c r="B10340" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10340" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10341" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10341" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10341" s="21"/>
+      <c r="C10341" s="22"/>
+    </row>
   </sheetData>
-  <mergeCells count="193">
+  <mergeCells count="211">
+    <mergeCell ref="C10158:C10159"/>
+    <mergeCell ref="C10217:C10218"/>
+    <mergeCell ref="B10336:B10337"/>
+    <mergeCell ref="C10338:C10339"/>
+    <mergeCell ref="C9916:C9917"/>
+    <mergeCell ref="C10276:C10277"/>
+    <mergeCell ref="C9870:C9871"/>
+    <mergeCell ref="B9868:B9869"/>
+    <mergeCell ref="C9977:C9978"/>
+    <mergeCell ref="C10034:C10035"/>
+    <mergeCell ref="C9564:C9565"/>
+    <mergeCell ref="C9627:C9628"/>
+    <mergeCell ref="C9686:C9687"/>
+    <mergeCell ref="C9745:C9746"/>
+    <mergeCell ref="C9804:C9805"/>
     <mergeCell ref="C9149:C9150"/>
     <mergeCell ref="B9276:B9277"/>
     <mergeCell ref="B9335:B9336"/>
     <mergeCell ref="B9394:B9395"/>
+    <mergeCell ref="C9446:C9447"/>
+    <mergeCell ref="B9498:C9498"/>
+    <mergeCell ref="C9516:C9517"/>
     <mergeCell ref="B8926:B8927"/>
     <mergeCell ref="B8908:C8908"/>
     <mergeCell ref="C8972:C8973"/>

</xml_diff>

<commit_message>
Instructions up to C1.
</commit_message>
<xml_diff>
--- a/Research/Instructions/Instructions Native SNES.xlsx
+++ b/Research/Instructions/Instructions Native SNES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Projects\BirdSNES\Research\Instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36DB2B1A-1CD9-4765-8CEA-188692191B7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11EB1F10-CC1C-4A21-8764-122D08C3B3A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$10381</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$11325</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4800" uniqueCount="481">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5205" uniqueCount="505">
   <si>
     <t>BRK (00)</t>
   </si>
@@ -15377,6 +15377,907 @@
   </si>
   <si>
     <t>LDA (AF)</t>
+  </si>
+  <si>
+    <t>Direct, Y (Write)</t>
+  </si>
+  <si>
+    <t>BCS (B0)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Inc. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Decide to branch if </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is 1.</t>
+    </r>
+  </si>
+  <si>
+    <t>LDA (B1)</t>
+  </si>
+  <si>
+    <t>LDA (B2)</t>
+  </si>
+  <si>
+    <t>LDA (B3)</t>
+  </si>
+  <si>
+    <t>LDY (B4)</t>
+  </si>
+  <si>
+    <t>LDA (B5)</t>
+  </si>
+  <si>
+    <t>LDX (B6)</t>
+  </si>
+  <si>
+    <t>Direct, Y (Read)</t>
+  </si>
+  <si>
+    <t>LDA (B7)</t>
+  </si>
+  <si>
+    <t>CLV (B8)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Sets the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>V</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag to 0.</t>
+    </r>
+  </si>
+  <si>
+    <t>LDA (B9)</t>
+  </si>
+  <si>
+    <t>Inc. PC. Perform Orig = Pointer.</t>
+  </si>
+  <si>
+    <t>TSX (BA)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">If </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag is set, perform </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L = </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L &amp; $80), and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L, otherwise perform </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> = </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.H &amp; $80), and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>TYX (BB)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">If </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag is set, perform </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L = </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L &amp; $80), and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L, otherwise perform </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> = </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.H &amp; $80), and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>LDY (BC)</t>
+  </si>
+  <si>
+    <t>LDA (BD)</t>
+  </si>
+  <si>
+    <t>LDX (BE)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">If </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag is set, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L to Operand.L, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L &amp; $80), and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off X.L, otherwise set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to Operand, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.H &amp; $80), and set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>LDA (BF)</t>
   </si>
 </sst>
 </file>
@@ -15990,7 +16891,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{236A51FB-68FA-4644-A8C6-D47AA32EBCC5}">
-  <dimension ref="A1:C10341"/>
+  <dimension ref="A1:C11287"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25.7109375" customWidth="1"/>
@@ -43780,7 +44681,7 @@
     <row r="8849" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8849" s="4"/>
       <c r="B8849" s="26" t="s">
-        <v>358</v>
+        <v>481</v>
       </c>
       <c r="C8849" s="27"/>
     </row>
@@ -47517,8 +48418,2715 @@
       <c r="B10341" s="21"/>
       <c r="C10341" s="22"/>
     </row>
+    <row r="10382" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10382" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="B10382" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10382" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10383" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10383" s="4"/>
+      <c r="B10383" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="C10383" s="6"/>
+    </row>
+    <row r="10384" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10384" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10384" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10384" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10385" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10385" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10385" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10385" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10386" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10386" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B10386" s="9"/>
+      <c r="C10386" s="10" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="10387" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10387" s="19">
+        <v>1.2</v>
+      </c>
+      <c r="B10387" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10387" s="10" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="10388" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10388" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B10388" s="9"/>
+      <c r="C10388" s="10" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="10389" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10389" s="19">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B10389" s="9"/>
+      <c r="C10389" s="10" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="10390" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10390" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B10390" s="9"/>
+      <c r="C10390" s="10" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="10391" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10391" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B10391" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10391" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10392" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10392" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10392" s="21"/>
+      <c r="C10392" s="22"/>
+    </row>
+    <row r="10441" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10441" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="B10441" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10441" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10442" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10442" s="4"/>
+      <c r="B10442" s="34" t="s">
+        <v>125</v>
+      </c>
+      <c r="C10442" s="35"/>
+    </row>
+    <row r="10443" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10443" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10443" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10443" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10444" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10444" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10444" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10444" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10445" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10445" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B10445" s="9"/>
+      <c r="C10445" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10446" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10446" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B10446" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10446" s="10" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="10447" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10447" s="16">
+        <v>2.1</v>
+      </c>
+      <c r="B10447" s="17"/>
+      <c r="C10447" s="24" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10448" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10448" s="16">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B10448" s="17"/>
+      <c r="C10448" s="24"/>
+    </row>
+    <row r="10449" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10449" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B10449" s="9"/>
+      <c r="C10449" s="10" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="10450" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10450" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B10450" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10450" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10451" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10451" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B10451" s="9"/>
+      <c r="C10451" s="10"/>
+    </row>
+    <row r="10452" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10452" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B10452" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10452" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10453" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10453" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B10453" s="9"/>
+      <c r="C10453" s="10" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="10454" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10454" s="8"/>
+      <c r="B10454" s="9"/>
+      <c r="C10454" s="10" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="10455" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10455" s="8"/>
+      <c r="B10455" s="9"/>
+      <c r="C10455" s="10" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="10456" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10456" s="8"/>
+      <c r="B10456" s="9"/>
+      <c r="C10456" s="10" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="10457" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10457" s="8"/>
+      <c r="B10457" s="9"/>
+      <c r="C10457" s="10" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="10458" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10458" s="16">
+        <v>5.2</v>
+      </c>
+      <c r="B10458" s="17"/>
+      <c r="C10458" s="24"/>
+    </row>
+    <row r="10459" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10459" s="16">
+        <v>6.1</v>
+      </c>
+      <c r="B10459" s="17"/>
+      <c r="C10459" s="24"/>
+    </row>
+    <row r="10460" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10460" s="19">
+        <v>6.2</v>
+      </c>
+      <c r="B10460" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C10460" s="10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10461" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10461" s="16">
+        <v>7.1</v>
+      </c>
+      <c r="B10461" s="17"/>
+      <c r="C10461" s="24"/>
+    </row>
+    <row r="10462" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10462" s="25">
+        <v>7.2</v>
+      </c>
+      <c r="B10462" s="33" t="s">
+        <v>349</v>
+      </c>
+      <c r="C10462" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10463" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10463" s="25"/>
+      <c r="B10463" s="33"/>
+      <c r="C10463" s="24"/>
+    </row>
+    <row r="10464" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10464" s="8">
+        <v>8.1</v>
+      </c>
+      <c r="B10464" s="9"/>
+      <c r="C10464" s="36" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="10465" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10465" s="8"/>
+      <c r="B10465" s="9"/>
+      <c r="C10465" s="36"/>
+    </row>
+    <row r="10466" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10466" s="8">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="B10466" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10466" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10467" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10467" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10467" s="21"/>
+      <c r="C10467" s="22"/>
+    </row>
+    <row r="10500" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10500" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="B10500" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10500" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10501" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10501" s="4"/>
+      <c r="B10501" s="26" t="s">
+        <v>127</v>
+      </c>
+      <c r="C10501" s="27"/>
+    </row>
+    <row r="10502" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10502" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10502" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10502" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10503" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10503" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10503" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10503" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10504" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10504" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B10504" s="9"/>
+      <c r="C10504" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10505" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10505" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B10505" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10505" s="10" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="10506" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10506" s="16">
+        <v>2.1</v>
+      </c>
+      <c r="B10506" s="17"/>
+      <c r="C10506" s="24" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10507" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10507" s="16">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B10507" s="17"/>
+      <c r="C10507" s="24"/>
+    </row>
+    <row r="10508" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10508" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B10508" s="9"/>
+      <c r="C10508" s="10" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="10509" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10509" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B10509" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10509" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10510" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10510" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B10510" s="9"/>
+      <c r="C10510" s="10"/>
+    </row>
+    <row r="10511" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10511" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B10511" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10511" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10512" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10512" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B10512" s="9"/>
+      <c r="C10512" s="10"/>
+    </row>
+    <row r="10513" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10513" s="19">
+        <v>5.2</v>
+      </c>
+      <c r="B10513" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C10513" s="10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10514" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10514" s="16">
+        <v>6.1</v>
+      </c>
+      <c r="B10514" s="17"/>
+      <c r="C10514" s="24"/>
+    </row>
+    <row r="10515" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10515" s="25">
+        <v>6.2</v>
+      </c>
+      <c r="B10515" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="C10515" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10516" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10516" s="8">
+        <v>7.1</v>
+      </c>
+      <c r="B10516" s="9"/>
+      <c r="C10516" s="36" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="10517" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10517" s="8"/>
+      <c r="B10517" s="9"/>
+      <c r="C10517" s="36"/>
+    </row>
+    <row r="10518" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10518" s="8">
+        <v>7.2</v>
+      </c>
+      <c r="B10518" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10518" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10519" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10519" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10519" s="21"/>
+      <c r="C10519" s="22"/>
+    </row>
+    <row r="10559" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10559" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="B10559" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C10559" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10560" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10560" s="4"/>
+      <c r="B10560" s="34" t="s">
+        <v>130</v>
+      </c>
+      <c r="C10560" s="35"/>
+    </row>
+    <row r="10561" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10561" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10561" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10561" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10562" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10562" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10562" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10562" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10563" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10563" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B10563" s="9"/>
+      <c r="C10563" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10564" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10564" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B10564" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10564" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10565" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10565" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B10565" s="9"/>
+      <c r="C10565" s="10" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="10566" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10566" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B10566" s="9"/>
+      <c r="C10566" s="10"/>
+    </row>
+    <row r="10567" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10567" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B10567" s="9"/>
+      <c r="C10567" s="10"/>
+    </row>
+    <row r="10568" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10568" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B10568" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10568" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10569" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10569" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B10569" s="9"/>
+      <c r="C10569" s="10"/>
+    </row>
+    <row r="10570" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10570" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B10570" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10570" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10571" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10571" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B10571" s="9"/>
+      <c r="C10571" s="10" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="10572" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10572" s="8"/>
+      <c r="B10572" s="9"/>
+      <c r="C10572" s="10" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="10573" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10573" s="8"/>
+      <c r="B10573" s="9"/>
+      <c r="C10573" s="10" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="10574" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10574" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="B10574" s="9"/>
+      <c r="C10574" s="10"/>
+    </row>
+    <row r="10575" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10575" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="B10575" s="9"/>
+      <c r="C10575" s="10"/>
+    </row>
+    <row r="10576" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10576" s="19">
+        <v>6.2</v>
+      </c>
+      <c r="B10576" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C10576" s="10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10577" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10577" s="16">
+        <v>7.1</v>
+      </c>
+      <c r="B10577" s="17"/>
+      <c r="C10577" s="24"/>
+    </row>
+    <row r="10578" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10578" s="25">
+        <v>7.2</v>
+      </c>
+      <c r="B10578" s="33" t="s">
+        <v>349</v>
+      </c>
+      <c r="C10578" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10579" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10579" s="25"/>
+      <c r="B10579" s="33"/>
+      <c r="C10579" s="24"/>
+    </row>
+    <row r="10580" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10580" s="8">
+        <v>8.1</v>
+      </c>
+      <c r="B10580" s="9"/>
+      <c r="C10580" s="36" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="10581" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10581" s="8"/>
+      <c r="B10581" s="9"/>
+      <c r="C10581" s="36"/>
+    </row>
+    <row r="10582" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10582" s="8">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="B10582" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10582" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10583" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10583" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10583" s="21"/>
+      <c r="C10583" s="22"/>
+    </row>
+    <row r="10618" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10618" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="B10618" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10618" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10619" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10619" s="4"/>
+      <c r="B10619" s="26" t="s">
+        <v>137</v>
+      </c>
+      <c r="C10619" s="27"/>
+    </row>
+    <row r="10620" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10620" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10620" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10620" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10621" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10621" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10621" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10621" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10622" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10622" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B10622" s="9"/>
+      <c r="C10622" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10623" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10623" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B10623" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10623" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10624" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10624" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B10624" s="9"/>
+      <c r="C10624" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10625" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10625" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B10625" s="9"/>
+      <c r="C10625" s="10"/>
+    </row>
+    <row r="10626" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10626" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B10626" s="9"/>
+      <c r="C10626" s="10" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="10627" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10627" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B10627" s="9"/>
+      <c r="C10627" s="10"/>
+    </row>
+    <row r="10628" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10628" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B10628" s="9"/>
+      <c r="C10628" s="10"/>
+    </row>
+    <row r="10629" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10629" s="19">
+        <v>4.2</v>
+      </c>
+      <c r="B10629" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10629" s="10" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="10630" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10630" s="16">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B10630" s="17"/>
+      <c r="C10630" s="24"/>
+    </row>
+    <row r="10631" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10631" s="25">
+        <v>5.2</v>
+      </c>
+      <c r="B10631" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10631" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10632" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10632" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="B10632" s="9"/>
+      <c r="C10632" s="36" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="10633" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10633" s="8"/>
+      <c r="B10633" s="9"/>
+      <c r="C10633" s="36"/>
+    </row>
+    <row r="10634" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10634" s="8">
+        <v>6.2</v>
+      </c>
+      <c r="B10634" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10634" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10635" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10635" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10635" s="21"/>
+      <c r="C10635" s="22"/>
+    </row>
+    <row r="10677" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10677" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="B10677" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10677" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10678" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10678" s="4"/>
+      <c r="B10678" s="26" t="s">
+        <v>137</v>
+      </c>
+      <c r="C10678" s="27"/>
+    </row>
+    <row r="10679" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10679" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10679" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10679" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10680" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10680" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10680" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10680" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10681" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10681" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B10681" s="9"/>
+      <c r="C10681" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10682" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10682" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B10682" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10682" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10683" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10683" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B10683" s="9"/>
+      <c r="C10683" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10684" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10684" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B10684" s="9"/>
+      <c r="C10684" s="10"/>
+    </row>
+    <row r="10685" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10685" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B10685" s="9"/>
+      <c r="C10685" s="10" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="10686" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10686" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B10686" s="9"/>
+      <c r="C10686" s="10"/>
+    </row>
+    <row r="10687" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10687" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B10687" s="9"/>
+      <c r="C10687" s="10"/>
+    </row>
+    <row r="10688" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10688" s="19">
+        <v>4.2</v>
+      </c>
+      <c r="B10688" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10688" s="10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10689" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10689" s="16">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B10689" s="17"/>
+      <c r="C10689" s="24"/>
+    </row>
+    <row r="10690" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10690" s="25">
+        <v>5.2</v>
+      </c>
+      <c r="B10690" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10690" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10691" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10691" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="B10691" s="9"/>
+      <c r="C10691" s="36" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="10692" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10692" s="8"/>
+      <c r="B10692" s="9"/>
+      <c r="C10692" s="36"/>
+    </row>
+    <row r="10693" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10693" s="8">
+        <v>6.2</v>
+      </c>
+      <c r="B10693" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10693" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10694" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10694" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10694" s="21"/>
+      <c r="C10694" s="22"/>
+    </row>
+    <row r="10736" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10736" s="1" t="s">
+        <v>489</v>
+      </c>
+      <c r="B10736" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10736" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10737" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10737" s="4"/>
+      <c r="B10737" s="26" t="s">
+        <v>490</v>
+      </c>
+      <c r="C10737" s="27"/>
+    </row>
+    <row r="10738" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10738" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10738" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10738" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10739" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10739" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10739" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10739" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10740" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10740" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B10740" s="9"/>
+      <c r="C10740" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10741" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10741" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B10741" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10741" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10742" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10742" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B10742" s="9"/>
+      <c r="C10742" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10743" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10743" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B10743" s="9"/>
+      <c r="C10743" s="10"/>
+    </row>
+    <row r="10744" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10744" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B10744" s="9"/>
+      <c r="C10744" s="10" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="10745" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10745" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B10745" s="9"/>
+      <c r="C10745" s="10"/>
+    </row>
+    <row r="10746" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10746" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B10746" s="9"/>
+      <c r="C10746" s="10"/>
+    </row>
+    <row r="10747" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10747" s="19">
+        <v>4.2</v>
+      </c>
+      <c r="B10747" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10747" s="10" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="10748" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10748" s="16">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B10748" s="17"/>
+      <c r="C10748" s="24"/>
+    </row>
+    <row r="10749" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10749" s="25">
+        <v>5.2</v>
+      </c>
+      <c r="B10749" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10749" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10750" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10750" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="B10750" s="9"/>
+      <c r="C10750" s="36" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="10751" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10751" s="8"/>
+      <c r="B10751" s="9"/>
+      <c r="C10751" s="36"/>
+    </row>
+    <row r="10752" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10752" s="8">
+        <v>6.2</v>
+      </c>
+      <c r="B10752" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10752" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10753" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10753" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10753" s="21"/>
+      <c r="C10753" s="22"/>
+    </row>
+    <row r="10795" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10795" s="1" t="s">
+        <v>491</v>
+      </c>
+      <c r="B10795" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10795" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10796" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10796" s="4"/>
+      <c r="B10796" s="34" t="s">
+        <v>142</v>
+      </c>
+      <c r="C10796" s="35"/>
+    </row>
+    <row r="10797" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10797" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10797" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10797" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10798" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10798" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10798" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10798" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10799" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10799" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B10799" s="9"/>
+      <c r="C10799" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10800" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10800" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B10800" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10800" s="10" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="10801" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10801" s="16">
+        <v>2.1</v>
+      </c>
+      <c r="B10801" s="17"/>
+      <c r="C10801" s="24" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10802" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10802" s="16">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B10802" s="17"/>
+      <c r="C10802" s="24"/>
+    </row>
+    <row r="10803" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10803" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B10803" s="9"/>
+      <c r="C10803" s="10" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="10804" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10804" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B10804" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10804" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10805" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10805" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B10805" s="9"/>
+      <c r="C10805" s="10"/>
+    </row>
+    <row r="10806" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10806" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B10806" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10806" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10807" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10807" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B10807" s="9"/>
+      <c r="C10807" s="10"/>
+    </row>
+    <row r="10808" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10808" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="B10808" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="C10808" s="10" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="10809" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10809" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="B10809" s="9"/>
+      <c r="C10809" s="10" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="10810" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10810" s="8"/>
+      <c r="B10810" s="9"/>
+      <c r="C10810" s="10" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="10811" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10811" s="8"/>
+      <c r="B10811" s="9"/>
+      <c r="C10811" s="10" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="10812" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10812" s="19">
+        <v>6.2</v>
+      </c>
+      <c r="B10812" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C10812" s="10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10813" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10813" s="16">
+        <v>7.1</v>
+      </c>
+      <c r="B10813" s="17"/>
+      <c r="C10813" s="24"/>
+    </row>
+    <row r="10814" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10814" s="25">
+        <v>7.2</v>
+      </c>
+      <c r="B10814" s="33" t="s">
+        <v>349</v>
+      </c>
+      <c r="C10814" s="18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10815" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10815" s="25"/>
+      <c r="B10815" s="33"/>
+      <c r="C10815" s="18"/>
+    </row>
+    <row r="10816" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10816" s="8">
+        <v>8.1</v>
+      </c>
+      <c r="B10816" s="9"/>
+      <c r="C10816" s="36" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="10817" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10817" s="8"/>
+      <c r="B10817" s="9"/>
+      <c r="C10817" s="36"/>
+    </row>
+    <row r="10818" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10818" s="8">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="B10818" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10818" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10819" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10819" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10819" s="21"/>
+      <c r="C10819" s="22"/>
+    </row>
+    <row r="10854" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10854" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="B10854" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10854" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10855" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10855" s="4"/>
+      <c r="B10855" s="26" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10855" s="27"/>
+    </row>
+    <row r="10856" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10856" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10856" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10856" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10857" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10857" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10857" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10857" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10858" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10858" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B10858" s="9"/>
+      <c r="C10858" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10859" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10859" s="19">
+        <v>1.2</v>
+      </c>
+      <c r="B10859" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10859" s="10" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="10860" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10860" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B10860" s="9"/>
+      <c r="C10860" s="10" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="10861" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10861" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B10861" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10861" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10862" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10862" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10862" s="21"/>
+      <c r="C10862" s="22"/>
+    </row>
+    <row r="10913" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10913" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="B10913" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10913" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10914" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10914" s="4"/>
+      <c r="B10914" s="26" t="s">
+        <v>146</v>
+      </c>
+      <c r="C10914" s="27"/>
+    </row>
+    <row r="10915" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10915" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10915" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10915" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10916" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10916" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10916" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10916" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10917" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10917" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B10917" s="9"/>
+      <c r="C10917" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10918" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10918" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B10918" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10918" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10919" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10919" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B10919" s="9"/>
+      <c r="C10919" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10920" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10920" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B10920" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10920" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10921" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10921" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B10921" s="9"/>
+      <c r="C10921" s="10" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="10922" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10922" s="8"/>
+      <c r="B10922" s="9"/>
+      <c r="C10922" s="10" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="10923" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10923" s="8"/>
+      <c r="B10923" s="9"/>
+      <c r="C10923" s="10" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="10924" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10924" s="8"/>
+      <c r="B10924" s="9"/>
+      <c r="C10924" s="10" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="10925" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10925" s="8"/>
+      <c r="B10925" s="9"/>
+      <c r="C10925" s="10" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="10926" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10926" s="16">
+        <v>3.2</v>
+      </c>
+      <c r="B10926" s="17"/>
+      <c r="C10926" s="24"/>
+    </row>
+    <row r="10927" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10927" s="16">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B10927" s="17"/>
+      <c r="C10927" s="24"/>
+    </row>
+    <row r="10928" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10928" s="19">
+        <v>4.2</v>
+      </c>
+      <c r="B10928" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C10928" s="10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10929" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10929" s="16">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B10929" s="17"/>
+      <c r="C10929" s="24"/>
+    </row>
+    <row r="10930" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10930" s="25">
+        <v>5.2</v>
+      </c>
+      <c r="B10930" s="33" t="s">
+        <v>349</v>
+      </c>
+      <c r="C10930" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10931" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10931" s="25"/>
+      <c r="B10931" s="33"/>
+      <c r="C10931" s="24"/>
+    </row>
+    <row r="10932" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10932" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="B10932" s="9"/>
+      <c r="C10932" s="36" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="10933" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10933" s="8"/>
+      <c r="B10933" s="9"/>
+      <c r="C10933" s="36"/>
+    </row>
+    <row r="10934" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10934" s="8">
+        <v>6.2</v>
+      </c>
+      <c r="B10934" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10934" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10935" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10935" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10935" s="21"/>
+      <c r="C10935" s="22"/>
+    </row>
+    <row r="10972" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10972" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="B10972" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10972" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10973" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10973" s="4"/>
+      <c r="B10973" s="26" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10973" s="27"/>
+    </row>
+    <row r="10974" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10974" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10974" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10974" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10975" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10975" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10975" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10975" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10976" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10976" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B10976" s="9"/>
+      <c r="C10976" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10977" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10977" s="19">
+        <v>1.2</v>
+      </c>
+      <c r="B10977" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10977" s="10" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="10978" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10978" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B10978" s="9"/>
+      <c r="C10978" s="36" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="10979" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10979" s="8"/>
+      <c r="B10979" s="9"/>
+      <c r="C10979" s="36"/>
+    </row>
+    <row r="10980" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10980" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B10980" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10980" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10981" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10981" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10981" s="21"/>
+      <c r="C10981" s="22"/>
+    </row>
+    <row r="11031" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11031" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="B11031" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11031" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11032" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11032" s="4"/>
+      <c r="B11032" s="26" t="s">
+        <v>1</v>
+      </c>
+      <c r="C11032" s="27"/>
+    </row>
+    <row r="11033" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11033" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11033" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11033" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11034" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11034" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11034" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11034" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11035" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11035" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B11035" s="9"/>
+      <c r="C11035" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11036" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11036" s="19">
+        <v>1.2</v>
+      </c>
+      <c r="B11036" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11036" s="10" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="11037" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11037" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B11037" s="9"/>
+      <c r="C11037" s="36" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="11038" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11038" s="8"/>
+      <c r="B11038" s="9"/>
+      <c r="C11038" s="36"/>
+    </row>
+    <row r="11039" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11039" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B11039" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11039" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11040" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11040" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11040" s="21"/>
+      <c r="C11040" s="22"/>
+    </row>
+    <row r="11090" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11090" s="1" t="s">
+        <v>500</v>
+      </c>
+      <c r="B11090" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11090" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11091" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11091" s="4"/>
+      <c r="B11091" s="26" t="s">
+        <v>155</v>
+      </c>
+      <c r="C11091" s="27"/>
+    </row>
+    <row r="11092" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11092" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11092" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11092" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11093" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11093" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11093" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11093" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11094" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11094" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B11094" s="9"/>
+      <c r="C11094" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11095" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11095" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B11095" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11095" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11096" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11096" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B11096" s="9"/>
+      <c r="C11096" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11097" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11097" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B11097" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11097" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11098" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11098" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B11098" s="9"/>
+      <c r="C11098" s="10" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="11099" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11099" s="8"/>
+      <c r="B11099" s="9"/>
+      <c r="C11099" s="10" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="11100" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11100" s="8"/>
+      <c r="B11100" s="9"/>
+      <c r="C11100" s="10" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="11101" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11101" s="8"/>
+      <c r="B11101" s="9"/>
+      <c r="C11101" s="10" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="11102" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11102" s="8"/>
+      <c r="B11102" s="9"/>
+      <c r="C11102" s="10" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="11103" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11103" s="16">
+        <v>3.2</v>
+      </c>
+      <c r="B11103" s="17"/>
+      <c r="C11103" s="24"/>
+    </row>
+    <row r="11104" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11104" s="16">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B11104" s="17"/>
+      <c r="C11104" s="24"/>
+    </row>
+    <row r="11105" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11105" s="19">
+        <v>4.2</v>
+      </c>
+      <c r="B11105" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C11105" s="10" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="11106" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11106" s="16">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B11106" s="17"/>
+      <c r="C11106" s="24"/>
+    </row>
+    <row r="11107" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11107" s="25">
+        <v>5.2</v>
+      </c>
+      <c r="B11107" s="33" t="s">
+        <v>349</v>
+      </c>
+      <c r="C11107" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11108" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11108" s="25"/>
+      <c r="B11108" s="33"/>
+      <c r="C11108" s="24"/>
+    </row>
+    <row r="11109" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11109" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="B11109" s="32"/>
+      <c r="C11109" s="36" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="11110" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11110" s="8"/>
+      <c r="B11110" s="32"/>
+      <c r="C11110" s="36"/>
+    </row>
+    <row r="11111" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11111" s="8">
+        <v>6.2</v>
+      </c>
+      <c r="B11111" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11111" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11112" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11112" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11112" s="21"/>
+      <c r="C11112" s="22"/>
+    </row>
+    <row r="11149" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11149" s="1" t="s">
+        <v>501</v>
+      </c>
+      <c r="B11149" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11149" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11150" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11150" s="4"/>
+      <c r="B11150" s="26" t="s">
+        <v>155</v>
+      </c>
+      <c r="C11150" s="27"/>
+    </row>
+    <row r="11151" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11151" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11151" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11151" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11152" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11152" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11152" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11152" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11153" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11153" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B11153" s="9"/>
+      <c r="C11153" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11154" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11154" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B11154" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11154" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11155" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11155" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B11155" s="9"/>
+      <c r="C11155" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11156" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11156" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B11156" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11156" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11157" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11157" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B11157" s="9"/>
+      <c r="C11157" s="10" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="11158" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11158" s="8"/>
+      <c r="B11158" s="9"/>
+      <c r="C11158" s="10" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="11159" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11159" s="8"/>
+      <c r="B11159" s="9"/>
+      <c r="C11159" s="10" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="11160" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11160" s="8"/>
+      <c r="B11160" s="9"/>
+      <c r="C11160" s="10" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="11161" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11161" s="8"/>
+      <c r="B11161" s="9"/>
+      <c r="C11161" s="10" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="11162" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11162" s="16">
+        <v>3.2</v>
+      </c>
+      <c r="B11162" s="17"/>
+      <c r="C11162" s="24"/>
+    </row>
+    <row r="11163" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11163" s="16">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B11163" s="17"/>
+      <c r="C11163" s="24"/>
+    </row>
+    <row r="11164" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11164" s="19">
+        <v>4.2</v>
+      </c>
+      <c r="B11164" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C11164" s="10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11165" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11165" s="16">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B11165" s="17"/>
+      <c r="C11165" s="24"/>
+    </row>
+    <row r="11166" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11166" s="25">
+        <v>5.2</v>
+      </c>
+      <c r="B11166" s="33" t="s">
+        <v>349</v>
+      </c>
+      <c r="C11166" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11167" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11167" s="25"/>
+      <c r="B11167" s="33"/>
+      <c r="C11167" s="24"/>
+    </row>
+    <row r="11168" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11168" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="B11168" s="32"/>
+      <c r="C11168" s="36" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="11169" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11169" s="8"/>
+      <c r="B11169" s="32"/>
+      <c r="C11169" s="36"/>
+    </row>
+    <row r="11170" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11170" s="8">
+        <v>6.2</v>
+      </c>
+      <c r="B11170" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11170" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11171" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11171" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11171" s="21"/>
+      <c r="C11171" s="22"/>
+    </row>
+    <row r="11208" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11208" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="B11208" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11208" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11209" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11209" s="4"/>
+      <c r="B11209" s="26" t="s">
+        <v>146</v>
+      </c>
+      <c r="C11209" s="27"/>
+    </row>
+    <row r="11210" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11210" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11210" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11210" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11211" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11211" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11211" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11211" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11212" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11212" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B11212" s="9"/>
+      <c r="C11212" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11213" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11213" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B11213" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11213" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11214" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11214" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B11214" s="9"/>
+      <c r="C11214" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11215" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11215" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B11215" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11215" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11216" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11216" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B11216" s="9"/>
+      <c r="C11216" s="10" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="11217" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11217" s="8"/>
+      <c r="B11217" s="9"/>
+      <c r="C11217" s="10" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="11218" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11218" s="8"/>
+      <c r="B11218" s="9"/>
+      <c r="C11218" s="10" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="11219" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11219" s="8"/>
+      <c r="B11219" s="9"/>
+      <c r="C11219" s="10" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="11220" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11220" s="8"/>
+      <c r="B11220" s="9"/>
+      <c r="C11220" s="10" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="11221" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11221" s="16">
+        <v>3.2</v>
+      </c>
+      <c r="B11221" s="17"/>
+      <c r="C11221" s="24"/>
+    </row>
+    <row r="11222" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11222" s="16">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B11222" s="17"/>
+      <c r="C11222" s="24"/>
+    </row>
+    <row r="11223" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11223" s="19">
+        <v>4.2</v>
+      </c>
+      <c r="B11223" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C11223" s="10" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="11224" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11224" s="16">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B11224" s="17"/>
+      <c r="C11224" s="24"/>
+    </row>
+    <row r="11225" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11225" s="25">
+        <v>5.2</v>
+      </c>
+      <c r="B11225" s="33" t="s">
+        <v>349</v>
+      </c>
+      <c r="C11225" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11226" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11226" s="25"/>
+      <c r="B11226" s="33"/>
+      <c r="C11226" s="24"/>
+    </row>
+    <row r="11227" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11227" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="B11227" s="32"/>
+      <c r="C11227" s="36" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="11228" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11228" s="8"/>
+      <c r="B11228" s="32"/>
+      <c r="C11228" s="36"/>
+    </row>
+    <row r="11229" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11229" s="8">
+        <v>6.2</v>
+      </c>
+      <c r="B11229" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11229" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11230" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11230" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11230" s="21"/>
+      <c r="C11230" s="22"/>
+    </row>
+    <row r="11267" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11267" s="1" t="s">
+        <v>504</v>
+      </c>
+      <c r="B11267" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11267" s="3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="11268" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11268" s="4"/>
+      <c r="B11268" s="26" t="s">
+        <v>163</v>
+      </c>
+      <c r="C11268" s="27"/>
+    </row>
+    <row r="11269" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11269" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11269" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11269" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11270" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11270" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11270" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11270" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11271" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11271" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B11271" s="9"/>
+      <c r="C11271" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11272" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11272" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B11272" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11272" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11273" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11273" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B11273" s="9"/>
+      <c r="C11273" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11274" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11274" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B11274" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11274" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11275" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11275" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B11275" s="9"/>
+      <c r="C11275" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11276" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11276" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B11276" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11276" s="10" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="11277" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11277" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B11277" s="9"/>
+      <c r="C11277" s="10" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="11278" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11278" s="8"/>
+      <c r="B11278" s="9"/>
+      <c r="C11278" s="10" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="11279" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11279" s="8"/>
+      <c r="B11279" s="9"/>
+      <c r="C11279" s="10" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="11280" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11280" s="19">
+        <v>4.2</v>
+      </c>
+      <c r="B11280" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C11280" s="10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11281" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11281" s="16">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B11281" s="17"/>
+      <c r="C11281" s="24"/>
+    </row>
+    <row r="11282" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11282" s="25">
+        <v>5.2</v>
+      </c>
+      <c r="B11282" s="33" t="s">
+        <v>349</v>
+      </c>
+      <c r="C11282" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11283" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11283" s="25"/>
+      <c r="B11283" s="33"/>
+      <c r="C11283" s="24"/>
+    </row>
+    <row r="11284" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11284" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="B11284" s="9"/>
+      <c r="C11284" s="36" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="11285" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11285" s="8"/>
+      <c r="B11285" s="9"/>
+      <c r="C11285" s="36"/>
+    </row>
+    <row r="11286" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11286" s="8">
+        <v>6.2</v>
+      </c>
+      <c r="B11286" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11286" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11287" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11287" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11287" s="21"/>
+      <c r="C11287" s="22"/>
+    </row>
   </sheetData>
-  <mergeCells count="211">
+  <mergeCells count="236">
+    <mergeCell ref="B11166:B11167"/>
+    <mergeCell ref="C11168:C11169"/>
+    <mergeCell ref="B11225:B11226"/>
+    <mergeCell ref="C11227:C11228"/>
+    <mergeCell ref="B11282:B11283"/>
+    <mergeCell ref="C11284:C11285"/>
+    <mergeCell ref="B10930:B10931"/>
+    <mergeCell ref="C10932:C10933"/>
+    <mergeCell ref="C10978:C10979"/>
+    <mergeCell ref="C11037:C11038"/>
+    <mergeCell ref="B11107:B11108"/>
+    <mergeCell ref="C11109:C11110"/>
+    <mergeCell ref="C10816:C10817"/>
+    <mergeCell ref="B10814:B10815"/>
+    <mergeCell ref="B10796:C10796"/>
+    <mergeCell ref="B10578:B10579"/>
+    <mergeCell ref="C10580:C10581"/>
+    <mergeCell ref="C10632:C10633"/>
+    <mergeCell ref="C10691:C10692"/>
+    <mergeCell ref="C10750:C10751"/>
+    <mergeCell ref="B10462:B10463"/>
+    <mergeCell ref="C10464:C10465"/>
+    <mergeCell ref="B10442:C10442"/>
+    <mergeCell ref="C10516:C10517"/>
+    <mergeCell ref="B10560:C10560"/>
     <mergeCell ref="C10158:C10159"/>
     <mergeCell ref="C10217:C10218"/>
     <mergeCell ref="B10336:B10337"/>

</xml_diff>